<commit_message>
Add 15 new registrations (orders 3843-3861): rolls and admit cards; update send progress
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Admit_Card_Data_2026.xlsx
+++ b/Admit_Card_Data_2026.xlsx
@@ -14,11 +14,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Raw_Data" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Admit_Data'!$A$1:$M$270</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Admit_Data'!$A$1:$M$285</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Separate'!$A$1:$N$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Review'!$A$1:$D$44</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Review'!$A$1:$D$46</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Centre_Map'!$A$1:$C$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Raw_Data'!$A$1:$S$271</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Raw_Data'!$A$1:$S$286</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M270"/>
+  <dimension ref="A1:M285"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -16153,8 +16153,883 @@
         </is>
       </c>
     </row>
+    <row r="271">
+      <c r="A271" s="2" t="n">
+        <v>3843</v>
+      </c>
+      <c r="B271" s="2" t="inlineStr">
+        <is>
+          <t>41126048</t>
+        </is>
+      </c>
+      <c r="C271" s="2" t="inlineStr">
+        <is>
+          <t>Admit_41126048_Duplicate</t>
+        </is>
+      </c>
+      <c r="D271" s="2" t="inlineStr">
+        <is>
+          <t>Boy</t>
+        </is>
+      </c>
+      <c r="E271" s="2" t="inlineStr">
+        <is>
+          <t>Safwan Zaman Ahnaf</t>
+        </is>
+      </c>
+      <c r="F271" s="2" t="inlineStr">
+        <is>
+          <t>Md Shahiduzzaman</t>
+        </is>
+      </c>
+      <c r="G271" s="2" t="inlineStr">
+        <is>
+          <t>Delta School and College</t>
+        </is>
+      </c>
+      <c r="H271" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="I271" s="2" t="inlineStr">
+        <is>
+          <t>+8801850401816</t>
+        </is>
+      </c>
+      <c r="J271" s="2" t="inlineStr">
+        <is>
+          <t>Dewanhat</t>
+        </is>
+      </c>
+      <c r="K271" s="2" t="inlineStr">
+        <is>
+          <t>চট্টগ্রাম কলেজিয়েট স্কুল</t>
+        </is>
+      </c>
+      <c r="L271" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="M271" s="2" t="inlineStr">
+        <is>
+          <t>Duplicate of order 3561 (same name &amp; father, different mobile)</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="n">
+        <v>3844</v>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>83126042</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>Admit_83126042</t>
+        </is>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>Boy</t>
+        </is>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>Twasin Alam</t>
+        </is>
+      </c>
+      <c r="F272" t="inlineStr">
+        <is>
+          <t>Md. Khurshidul Alam</t>
+        </is>
+      </c>
+      <c r="G272" t="inlineStr">
+        <is>
+          <t>Chattogram Collegiate School</t>
+        </is>
+      </c>
+      <c r="H272" t="n">
+        <v>8</v>
+      </c>
+      <c r="I272" t="inlineStr">
+        <is>
+          <t>+8801815287418</t>
+        </is>
+      </c>
+      <c r="J272" t="inlineStr">
+        <is>
+          <t>Halishahar</t>
+        </is>
+      </c>
+      <c r="K272" t="inlineStr">
+        <is>
+          <t>সিলভার বেলস কিন্ডারগার্টেন এন্ড গার্লস হাই স্কুল</t>
+        </is>
+      </c>
+      <c r="L272" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="n">
+        <v>3846</v>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>71126054</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>Admit_71126054</t>
+        </is>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>Boy</t>
+        </is>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>Md.Ridowan Bin Arif</t>
+        </is>
+      </c>
+      <c r="F273" t="inlineStr">
+        <is>
+          <t>Md.Ariful Islam</t>
+        </is>
+      </c>
+      <c r="G273" t="inlineStr">
+        <is>
+          <t>মোঃ আরিফুল ইসলাম</t>
+        </is>
+      </c>
+      <c r="H273" t="n">
+        <v>7</v>
+      </c>
+      <c r="I273" t="inlineStr">
+        <is>
+          <t>+8801722966006</t>
+        </is>
+      </c>
+      <c r="J273" t="inlineStr">
+        <is>
+          <t>Dewanhat</t>
+        </is>
+      </c>
+      <c r="K273" t="inlineStr">
+        <is>
+          <t>চট্টগ্রাম কলেজিয়েট স্কুল</t>
+        </is>
+      </c>
+      <c r="L273" t="inlineStr">
+        <is>
+          <t>Seven</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="n">
+        <v>3847</v>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>51126060</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>Admit_51126060</t>
+        </is>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>Boy</t>
+        </is>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>AHMAD JAHEE</t>
+        </is>
+      </c>
+      <c r="F274" t="inlineStr">
+        <is>
+          <t>JALAL UDDIN</t>
+        </is>
+      </c>
+      <c r="G274" t="inlineStr">
+        <is>
+          <t>CHATTOGRAM COLLEGIATE SCHOOL</t>
+        </is>
+      </c>
+      <c r="H274" t="n">
+        <v>5</v>
+      </c>
+      <c r="I274" t="inlineStr">
+        <is>
+          <t>+8801626914730</t>
+        </is>
+      </c>
+      <c r="J274" t="inlineStr">
+        <is>
+          <t>Dewanhat</t>
+        </is>
+      </c>
+      <c r="K274" t="inlineStr">
+        <is>
+          <t>চট্টগ্রাম কলেজিয়েট স্কুল</t>
+        </is>
+      </c>
+      <c r="L274" t="inlineStr">
+        <is>
+          <t>FIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="n">
+        <v>3848</v>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>72226059</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>Admit_72226059</t>
+        </is>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>Girl</t>
+        </is>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>Nusrat Jahan</t>
+        </is>
+      </c>
+      <c r="F275" t="inlineStr">
+        <is>
+          <t>Mohammed Jafor Iqbal Talukder</t>
+        </is>
+      </c>
+      <c r="G275" t="inlineStr">
+        <is>
+          <t>CDDL Navy School</t>
+        </is>
+      </c>
+      <c r="H275" t="n">
+        <v>7</v>
+      </c>
+      <c r="I275" t="inlineStr">
+        <is>
+          <t>+8801336826867</t>
+        </is>
+      </c>
+      <c r="J275" t="inlineStr">
+        <is>
+          <t>Patenga</t>
+        </is>
+      </c>
+      <c r="K275" t="inlineStr">
+        <is>
+          <t>পতেঙ্গা উচ্চ বিদ্যালয়</t>
+        </is>
+      </c>
+      <c r="L275" t="inlineStr">
+        <is>
+          <t>07</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="n">
+        <v>3849</v>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>93126020</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>Admit_93126020</t>
+        </is>
+      </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>Boy</t>
+        </is>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>Md.Samiul Islam Alvi</t>
+        </is>
+      </c>
+      <c r="F276" t="inlineStr">
+        <is>
+          <t>Md Saiful Islam</t>
+        </is>
+      </c>
+      <c r="G276" t="inlineStr">
+        <is>
+          <t>Ispahani Public School And College</t>
+        </is>
+      </c>
+      <c r="H276" t="n">
+        <v>9</v>
+      </c>
+      <c r="I276" t="inlineStr">
+        <is>
+          <t>+8801717944271</t>
+        </is>
+      </c>
+      <c r="J276" t="inlineStr">
+        <is>
+          <t>Agrabad</t>
+        </is>
+      </c>
+      <c r="K276" t="inlineStr">
+        <is>
+          <t>সিলভার বেলস কিন্ডারগার্টেন এন্ড গার্লস হাই স্কুল</t>
+        </is>
+      </c>
+      <c r="L276" t="inlineStr">
+        <is>
+          <t>09</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="n">
+        <v>3850</v>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>61226058</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>Admit_61226058</t>
+        </is>
+      </c>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>Girl</t>
+        </is>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>Tasnia Farin Yusha</t>
+        </is>
+      </c>
+      <c r="F277" t="inlineStr">
+        <is>
+          <t>Mohammad Mojibul Hoque</t>
+        </is>
+      </c>
+      <c r="G277" t="inlineStr">
+        <is>
+          <t>Dr. Khastagir Govt. Girls High School</t>
+        </is>
+      </c>
+      <c r="H277" t="n">
+        <v>6</v>
+      </c>
+      <c r="I277" t="inlineStr">
+        <is>
+          <t>+8801970433883</t>
+        </is>
+      </c>
+      <c r="J277" t="inlineStr">
+        <is>
+          <t>Dewanhat</t>
+        </is>
+      </c>
+      <c r="K277" t="inlineStr">
+        <is>
+          <t>চট্টগ্রাম কলেজিয়েট স্কুল</t>
+        </is>
+      </c>
+      <c r="L277" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="n">
+        <v>3852</v>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>62126067</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>Admit_62126067</t>
+        </is>
+      </c>
+      <c r="D278" t="inlineStr">
+        <is>
+          <t>Boy</t>
+        </is>
+      </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>Prantik Barua Dhrubo</t>
+        </is>
+      </c>
+      <c r="F278" t="inlineStr">
+        <is>
+          <t>Dipak Barua</t>
+        </is>
+      </c>
+      <c r="G278" t="inlineStr">
+        <is>
+          <t>Green Bell School &amp; College</t>
+        </is>
+      </c>
+      <c r="H278" t="n">
+        <v>6</v>
+      </c>
+      <c r="I278" t="inlineStr">
+        <is>
+          <t>+8801612938480</t>
+        </is>
+      </c>
+      <c r="J278" t="inlineStr">
+        <is>
+          <t>Patenga</t>
+        </is>
+      </c>
+      <c r="K278" t="inlineStr">
+        <is>
+          <t>পতেঙ্গা উচ্চ বিদ্যালয়</t>
+        </is>
+      </c>
+      <c r="L278" t="inlineStr">
+        <is>
+          <t>Class Six</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="n">
+        <v>3853</v>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>71126055</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>Admit_71126055</t>
+        </is>
+      </c>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>Boy</t>
+        </is>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>MD.Rayhan Alam</t>
+        </is>
+      </c>
+      <c r="F279" t="inlineStr">
+        <is>
+          <t>Jahangir Alam</t>
+        </is>
+      </c>
+      <c r="G279" t="inlineStr">
+        <is>
+          <t>Chattogram Collegiate School, Chattogram</t>
+        </is>
+      </c>
+      <c r="H279" t="n">
+        <v>7</v>
+      </c>
+      <c r="I279" t="inlineStr">
+        <is>
+          <t>+8801851911435</t>
+        </is>
+      </c>
+      <c r="J279" t="inlineStr">
+        <is>
+          <t>Dewanhat</t>
+        </is>
+      </c>
+      <c r="K279" t="inlineStr">
+        <is>
+          <t>চট্টগ্রাম কলেজিয়েট স্কুল</t>
+        </is>
+      </c>
+      <c r="L279" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="n">
+        <v>3854</v>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>53226123</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>Admit_53226123</t>
+        </is>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>Girl</t>
+        </is>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>Fahmida khanom alifa</t>
+        </is>
+      </c>
+      <c r="F280" t="inlineStr">
+        <is>
+          <t>Ayub khan</t>
+        </is>
+      </c>
+      <c r="G280" t="inlineStr">
+        <is>
+          <t>South kattali pran hori model gov't primary school</t>
+        </is>
+      </c>
+      <c r="H280" t="n">
+        <v>5</v>
+      </c>
+      <c r="I280" t="inlineStr">
+        <is>
+          <t>+8801789865054</t>
+        </is>
+      </c>
+      <c r="J280" t="inlineStr">
+        <is>
+          <t>Halishahar</t>
+        </is>
+      </c>
+      <c r="K280" t="inlineStr">
+        <is>
+          <t>সিলভার বেলস কিন্ডারগার্টেন এন্ড গার্লস হাই স্কুল</t>
+        </is>
+      </c>
+      <c r="L280" t="inlineStr">
+        <is>
+          <t>Five</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="n">
+        <v>3856</v>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>73126050</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>Admit_73126050</t>
+        </is>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>Boy</t>
+        </is>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>Mosaidul Hossain Nihad</t>
+        </is>
+      </c>
+      <c r="F281" t="inlineStr">
+        <is>
+          <t>Moazzam Hossain Molla</t>
+        </is>
+      </c>
+      <c r="G281" t="inlineStr">
+        <is>
+          <t>Halishahar Cantonment Public School and College</t>
+        </is>
+      </c>
+      <c r="H281" t="n">
+        <v>7</v>
+      </c>
+      <c r="I281" t="inlineStr">
+        <is>
+          <t>+8801675271093</t>
+        </is>
+      </c>
+      <c r="J281" t="inlineStr">
+        <is>
+          <t>Halishahar</t>
+        </is>
+      </c>
+      <c r="K281" t="inlineStr">
+        <is>
+          <t>সিলভার বেলস কিন্ডারগার্টেন এন্ড গার্লস হাই স্কুল</t>
+        </is>
+      </c>
+      <c r="L281" t="inlineStr">
+        <is>
+          <t>Seven</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="n">
+        <v>3857</v>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>63226077</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>Admit_63226077</t>
+        </is>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>Girl</t>
+        </is>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>Junaira Farisha Islam</t>
+        </is>
+      </c>
+      <c r="F282" t="inlineStr">
+        <is>
+          <t>Me.Manirul Islam</t>
+        </is>
+      </c>
+      <c r="G282" t="inlineStr">
+        <is>
+          <t>HCPSC</t>
+        </is>
+      </c>
+      <c r="H282" t="n">
+        <v>6</v>
+      </c>
+      <c r="I282" t="inlineStr">
+        <is>
+          <t>+8801838518567</t>
+        </is>
+      </c>
+      <c r="J282" t="inlineStr">
+        <is>
+          <t>Halishahar</t>
+        </is>
+      </c>
+      <c r="K282" t="inlineStr">
+        <is>
+          <t>সিলভার বেলস কিন্ডারগার্টেন এন্ড গার্লস হাই স্কুল</t>
+        </is>
+      </c>
+      <c r="L282" t="inlineStr">
+        <is>
+          <t>Six</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="n">
+        <v>3858</v>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>43126087</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>Admit_43126087</t>
+        </is>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>Boy</t>
+        </is>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>Zain Riyasat Islam</t>
+        </is>
+      </c>
+      <c r="F283" t="inlineStr">
+        <is>
+          <t>Md.Manirul Islam</t>
+        </is>
+      </c>
+      <c r="G283" t="inlineStr">
+        <is>
+          <t>HCPSC</t>
+        </is>
+      </c>
+      <c r="H283" t="n">
+        <v>4</v>
+      </c>
+      <c r="I283" t="inlineStr">
+        <is>
+          <t>+8801838518567</t>
+        </is>
+      </c>
+      <c r="J283" t="inlineStr">
+        <is>
+          <t>Halishahar</t>
+        </is>
+      </c>
+      <c r="K283" t="inlineStr">
+        <is>
+          <t>সিলভার বেলস কিন্ডারগার্টেন এন্ড গার্লস হাই স্কুল</t>
+        </is>
+      </c>
+      <c r="L283" t="inlineStr">
+        <is>
+          <t>Four</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="n">
+        <v>3860</v>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>71226068</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>Admit_71226068</t>
+        </is>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>Girl</t>
+        </is>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>Olin Atfa</t>
+        </is>
+      </c>
+      <c r="F284" t="inlineStr">
+        <is>
+          <t>MD. YEASIN ARAFAT</t>
+        </is>
+      </c>
+      <c r="G284" t="inlineStr">
+        <is>
+          <t>GUL-E-ZAR BEGUM CITY CORP MUSLIM GIRLS HIGH SCHOOL</t>
+        </is>
+      </c>
+      <c r="H284" t="n">
+        <v>7</v>
+      </c>
+      <c r="I284" t="inlineStr">
+        <is>
+          <t>+8801866358979</t>
+        </is>
+      </c>
+      <c r="J284" t="inlineStr">
+        <is>
+          <t>Dewanhat</t>
+        </is>
+      </c>
+      <c r="K284" t="inlineStr">
+        <is>
+          <t>চট্টগ্রাম কলেজিয়েট স্কুল</t>
+        </is>
+      </c>
+      <c r="L284" t="inlineStr">
+        <is>
+          <t>Seven</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="n">
+        <v>3861</v>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>51126061</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>Admit_51126061</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>Boy</t>
+        </is>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>AFSAN NAZRUL AR-RAFI</t>
+        </is>
+      </c>
+      <c r="F285" t="inlineStr">
+        <is>
+          <t>MD. NAZRUL ISLAM</t>
+        </is>
+      </c>
+      <c r="G285" t="inlineStr">
+        <is>
+          <t>Ispahani Public School &amp; College</t>
+        </is>
+      </c>
+      <c r="H285" t="n">
+        <v>5</v>
+      </c>
+      <c r="I285" t="inlineStr">
+        <is>
+          <t>+8801953031941</t>
+        </is>
+      </c>
+      <c r="J285" t="inlineStr">
+        <is>
+          <t>Dewanhat</t>
+        </is>
+      </c>
+      <c r="K285" t="inlineStr">
+        <is>
+          <t>চট্টগ্রাম কলেজিয়েট স্কুল</t>
+        </is>
+      </c>
+      <c r="L285" t="inlineStr">
+        <is>
+          <t>Five</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M270"/>
+  <autoFilter ref="A1:M285"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -16328,7 +17203,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D44"/>
+  <dimension ref="A1:D46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -16461,7 +17336,7 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>3750</v>
+        <v>3843</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -16470,18 +17345,18 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>MOHAMMED MUHTASIM ISLAM</t>
+          <t>Safwan Zaman Ahnaf</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>same student as order 3506 - kept both, marked in file name</t>
+          <t>likely same student as order 3561 - kept, marked in file name</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>3506</v>
+        <v>3750</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -16495,27 +17370,27 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>same student as order 3750 - kept both, marked in file name</t>
+          <t>same student as order 3506 - kept both, marked in file name</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>3446</v>
+        <v>3506</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Student</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>মোহাম্মদ নুরুল ইসলাম</t>
+          <t>MOHAMMED MUHTASIM ISLAM</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>written in Bangla (kept as entered)</t>
+          <t>same student as order 3750 - kept both, marked in file name</t>
         </is>
       </c>
     </row>
@@ -16525,12 +17400,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ডাঃ খাস্তগীর সরকারি বালিকা উচ্চ বিদ্যালয়</t>
+          <t>মোহাম্মদ নুরুল ইসলাম</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -16541,7 +17416,7 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>3509</v>
+        <v>3446</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -16550,7 +17425,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>ফুলকি সহজপাঠ বিদ্যালয়</t>
+          <t>ডাঃ খাস্তগীর সরকারি বালিকা উচ্চ বিদ্যালয়</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -16561,16 +17436,16 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>3604</v>
+        <v>3509</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>মোঃ আনোয়ার হোসেন</t>
+          <t>ফুলকি সহজপাঠ বিদ্যালয়</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -16585,12 +17460,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>হালিশহর ক্যান্টনম্যান্ট পাবলিক স্কুল এন্ড কলেজ</t>
+          <t>মোঃ আনোয়ার হোসেন</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -16601,16 +17476,16 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>3639</v>
+        <v>3604</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>মোঃ আবু সায়েম</t>
+          <t>হালিশহর ক্যান্টনম্যান্ট পাবলিক স্কুল এন্ড কলেজ</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -16625,12 +17500,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>বিএএফ শাহীন কলেজ</t>
+          <t>মোঃ আবু সায়েম</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -16641,16 +17516,16 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>3642</v>
+        <v>3639</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>মনির হোসেন</t>
+          <t>বিএএফ শাহীন কলেজ</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -16665,12 +17540,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>বিএএফ শাহীন কলেজ</t>
+          <t>মনির হোসেন</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -16681,16 +17556,16 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>3643</v>
+        <v>3642</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>মো: রেজাউল করিম</t>
+          <t>বিএএফ শাহীন কলেজ</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -16705,12 +17580,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>বিএএফ শাহীন কলেজ</t>
+          <t>মো: রেজাউল করিম</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -16721,16 +17596,16 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>3649</v>
+        <v>3643</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>মোঃ নিজাম উদ্দিন</t>
+          <t>বিএএফ শাহীন কলেজ</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -16745,12 +17620,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>বাংলাদেশ নৌবাহিনী স্কুল এন্ড কলেজ, চট্টগ্রাম</t>
+          <t>মোঃ নিজাম উদ্দিন</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -16761,16 +17636,16 @@
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>3670</v>
+        <v>3649</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>জুলফিকার আলী মিঠু</t>
+          <t>বাংলাদেশ নৌবাহিনী স্কুল এন্ড কলেজ, চট্টগ্রাম</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -16785,12 +17660,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>বিএএফ শাহীন কলেজ</t>
+          <t>জুলফিকার আলী মিঠু</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -16801,7 +17676,7 @@
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>3680</v>
+        <v>3670</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -16810,7 +17685,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>বলুয়ারদীঘি সিটি কর্পোরেশন বালিকা উচ্চ বিদ্যালয়</t>
+          <t>বিএএফ শাহীন কলেজ</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -16821,16 +17696,16 @@
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>3697</v>
+        <v>3680</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>কাকন চক্রবর্তী</t>
+          <t>বলুয়ারদীঘি সিটি কর্পোরেশন বালিকা উচ্চ বিদ্যালয়</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -16845,12 +17720,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>মুসলিম এডুকেশন সোসাইটি উচ্চ বিদ্যালয়</t>
+          <t>কাকন চক্রবর্তী</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -16861,16 +17736,16 @@
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>3718</v>
+        <v>3697</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>মনির আহমদ</t>
+          <t>মুসলিম এডুকেশন সোসাইটি উচ্চ বিদ্যালয়</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -16885,12 +17760,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>হাটহাজারী আনোয়ারুল উলুম নোমানীয়া ফাজিল মাদ্রাসা</t>
+          <t>মনির আহমদ</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -16901,16 +17776,16 @@
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>3724</v>
+        <v>3718</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>মনিরুল হক</t>
+          <t>হাটহাজারী আনোয়ারুল উলুম নোমানীয়া ফাজিল মাদ্রাসা</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -16925,12 +17800,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>বাহমনিখীল সরকারি প্রাথমিক বিদ্যালয়</t>
+          <t>মনিরুল হক</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -16941,16 +17816,16 @@
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>3748</v>
+        <v>3724</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>আবু বক্কর সিদ্দিক</t>
+          <t>বাহমনিখীল সরকারি প্রাথমিক বিদ্যালয়</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -16965,12 +17840,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>হালিশহর ক্যান্টনমেন্ট পাবলিক স্কুল এন্ড কলেজ</t>
+          <t>আবু বক্কর সিদ্দিক</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -16981,16 +17856,16 @@
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>3770</v>
+        <v>3748</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>মোহাম্মদ রেজাউল করিম</t>
+          <t>হালিশহর ক্যান্টনমেন্ট পাবলিক স্কুল এন্ড কলেজ</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -17005,12 +17880,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>রেলওয়ে পাবলিক স্কুল এন্ড কলেজ</t>
+          <t>মোহাম্মদ রেজাউল করিম</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -17021,16 +17896,16 @@
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>3773</v>
+        <v>3770</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>মোহাম্মদ রেজাউল করিম</t>
+          <t>রেলওয়ে পাবলিক স্কুল এন্ড কলেজ</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -17045,12 +17920,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>সেন্ট্রাল পাবলিক স্কুল এন্ড কলেজ</t>
+          <t>মোহাম্মদ রেজাউল করিম</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -17061,16 +17936,16 @@
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>3796</v>
+        <v>3773</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>মোহাম্মদ নওশাদ ইকবাল</t>
+          <t>সেন্ট্রাল পাবলিক স্কুল এন্ড কলেজ</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -17085,12 +17960,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>ইস্পাহানি পাবলিক স্কুল এন্ড কলেজ, চট্টগ্রাম।</t>
+          <t>মোহাম্মদ নওশাদ ইকবাল</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -17101,16 +17976,16 @@
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>3797</v>
+        <v>3796</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>মোহাম্মদ নওশাদ ইকবাল</t>
+          <t>ইস্পাহানি পাবলিক স্কুল এন্ড কলেজ, চট্টগ্রাম।</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -17125,12 +18000,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>ইস্পাহানি পাবলিক স্কুল এন্ড কলেজ, চট্টগ্রাম।</t>
+          <t>মোহাম্মদ নওশাদ ইকবাল</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -17141,16 +18016,16 @@
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>3835</v>
+        <v>3797</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>মো ইউসুফ</t>
+          <t>ইস্পাহানি পাবলিক স্কুল এন্ড কলেজ, চট্টগ্রাম।</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -17165,12 +18040,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>সি এম পি স্কুল এন্ড কলেজ</t>
+          <t>মো ইউসুফ</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -17181,16 +18056,16 @@
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>3840</v>
+        <v>3835</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>শাহা জাহান</t>
+          <t>সি এম পি স্কুল এন্ড কলেজ</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -17205,22 +18080,62 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
+          <t>Fathers Name</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>শাহা জাহান</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>written in Bangla (kept as entered)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>3840</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
           <t>Name of School</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
+      <c r="C45" t="inlineStr">
         <is>
           <t>বাকলিয়া আদর্শ বালিকা উচ্চ বিদ্যালয়</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr">
+      <c r="D45" t="inlineStr">
         <is>
           <t>written in Bangla (kept as entered)</t>
         </is>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>3846</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Name of School</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>মোঃ আরিফুল ইসলাম</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>written in Bangla (kept as entered)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D44"/>
+  <autoFilter ref="A1:D46"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -17268,7 +18183,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>129</v>
+        <v>136</v>
       </c>
     </row>
     <row r="3">
@@ -17283,7 +18198,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>78</v>
+        <v>83</v>
       </c>
     </row>
     <row r="4">
@@ -17298,7 +18213,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="5">
@@ -17313,7 +18228,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
   </sheetData>
@@ -17328,7 +18243,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S271"/>
+  <dimension ref="A1:S286"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -39574,8 +40489,1238 @@
         </is>
       </c>
     </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>3843</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>01720601933</t>
+        </is>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>DJE2WL950U</t>
+        </is>
+      </c>
+      <c r="G272" t="inlineStr">
+        <is>
+          <t>2026-10-14 07:18:02</t>
+        </is>
+      </c>
+      <c r="H272" t="inlineStr">
+        <is>
+          <t>Boy</t>
+        </is>
+      </c>
+      <c r="I272" t="inlineStr">
+        <is>
+          <t>Safwan Zaman Ahnaf</t>
+        </is>
+      </c>
+      <c r="J272" t="inlineStr">
+        <is>
+          <t>সাফওয়ান জামান আহনাফ</t>
+        </is>
+      </c>
+      <c r="K272" t="inlineStr">
+        <is>
+          <t>Md Shahiduzzaman</t>
+        </is>
+      </c>
+      <c r="L272" t="inlineStr">
+        <is>
+          <t>Tahmina Siddeka</t>
+        </is>
+      </c>
+      <c r="M272" t="inlineStr">
+        <is>
+          <t>Delta School and College</t>
+        </is>
+      </c>
+      <c r="N272" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="O272" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="P272" t="inlineStr">
+        <is>
+          <t>Bakolia Access Road, Bakolia, Chattogram</t>
+        </is>
+      </c>
+      <c r="Q272" t="inlineStr">
+        <is>
+          <t>01850401816</t>
+        </is>
+      </c>
+      <c r="S272" t="inlineStr">
+        <is>
+          <t>dewanhat</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>3844</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>01815287418</t>
+        </is>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>DJE90HFF6V</t>
+        </is>
+      </c>
+      <c r="G273" t="inlineStr">
+        <is>
+          <t>2026-10-14 16:12:02</t>
+        </is>
+      </c>
+      <c r="H273" t="inlineStr">
+        <is>
+          <t>Boy</t>
+        </is>
+      </c>
+      <c r="I273" t="inlineStr">
+        <is>
+          <t>Twasin Alam</t>
+        </is>
+      </c>
+      <c r="J273" t="inlineStr">
+        <is>
+          <t>ত্বসীন আলম</t>
+        </is>
+      </c>
+      <c r="K273" t="inlineStr">
+        <is>
+          <t>Md. Khurshidul Alam</t>
+        </is>
+      </c>
+      <c r="L273" t="inlineStr">
+        <is>
+          <t>Mst. Yesmin Akter</t>
+        </is>
+      </c>
+      <c r="M273" t="inlineStr">
+        <is>
+          <t>Chattogram Collegiate School</t>
+        </is>
+      </c>
+      <c r="N273" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="O273" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="P273" t="inlineStr">
+        <is>
+          <t>Nayabazar, Halishahar, Chattogram.</t>
+        </is>
+      </c>
+      <c r="Q273" t="inlineStr">
+        <is>
+          <t>01815287418</t>
+        </is>
+      </c>
+      <c r="S273" t="inlineStr">
+        <is>
+          <t>halishahar</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>3846</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>01722966006</t>
+        </is>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>DJF712IC31</t>
+        </is>
+      </c>
+      <c r="G274" t="inlineStr">
+        <is>
+          <t>2026-10-15 04:27:59</t>
+        </is>
+      </c>
+      <c r="H274" t="inlineStr">
+        <is>
+          <t>Boy</t>
+        </is>
+      </c>
+      <c r="I274" t="inlineStr">
+        <is>
+          <t>Md.Ridowan Bin Arif</t>
+        </is>
+      </c>
+      <c r="J274" t="inlineStr">
+        <is>
+          <t>মোঃ রিদওয়ান বিন আরিফ</t>
+        </is>
+      </c>
+      <c r="K274" t="inlineStr">
+        <is>
+          <t>Md.Ariful Islam</t>
+        </is>
+      </c>
+      <c r="L274" t="inlineStr">
+        <is>
+          <t>Rikta Akter</t>
+        </is>
+      </c>
+      <c r="M274" t="inlineStr">
+        <is>
+          <t>মোঃ আরিফুল ইসলাম</t>
+        </is>
+      </c>
+      <c r="N274" t="inlineStr">
+        <is>
+          <t>Seven</t>
+        </is>
+      </c>
+      <c r="O274" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="P274" t="inlineStr">
+        <is>
+          <t>Sadarghat, Chittagong</t>
+        </is>
+      </c>
+      <c r="Q274" t="inlineStr">
+        <is>
+          <t>01722966006</t>
+        </is>
+      </c>
+      <c r="S274" t="inlineStr">
+        <is>
+          <t>dewanhat</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>3847</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>01319004461</t>
+        </is>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>DJF01W6ENE</t>
+        </is>
+      </c>
+      <c r="G275" t="inlineStr">
+        <is>
+          <t>2026-10-15 12:38:55</t>
+        </is>
+      </c>
+      <c r="H275" t="inlineStr">
+        <is>
+          <t>Boy</t>
+        </is>
+      </c>
+      <c r="I275" t="inlineStr">
+        <is>
+          <t>AHMAD JAHEE</t>
+        </is>
+      </c>
+      <c r="J275" t="inlineStr">
+        <is>
+          <t>আহমাদ জাহী</t>
+        </is>
+      </c>
+      <c r="K275" t="inlineStr">
+        <is>
+          <t>JALAL UDDIN</t>
+        </is>
+      </c>
+      <c r="L275" t="inlineStr">
+        <is>
+          <t>SHAMIM AKTER</t>
+        </is>
+      </c>
+      <c r="M275" t="inlineStr">
+        <is>
+          <t>CHATTOGRAM COLLEGIATE SCHOOL</t>
+        </is>
+      </c>
+      <c r="N275" t="inlineStr">
+        <is>
+          <t>FIVE</t>
+        </is>
+      </c>
+      <c r="O275" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="P275" t="inlineStr">
+        <is>
+          <t>30 NO. M M ALI ROAD, LALKHAN BAZAR, VOTAIYA COLONY, DAMPARA-4000, KHULSHI, CHATTOGRAM</t>
+        </is>
+      </c>
+      <c r="Q275" t="inlineStr">
+        <is>
+          <t>01626914730</t>
+        </is>
+      </c>
+      <c r="S275" t="inlineStr">
+        <is>
+          <t>dewanhat</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>3848</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>01723088207</t>
+        </is>
+      </c>
+      <c r="F276" t="inlineStr">
+        <is>
+          <t>7659Q5GH</t>
+        </is>
+      </c>
+      <c r="G276" t="inlineStr">
+        <is>
+          <t>2026-10-15 13:33:41</t>
+        </is>
+      </c>
+      <c r="H276" t="inlineStr">
+        <is>
+          <t>Girl</t>
+        </is>
+      </c>
+      <c r="I276" t="inlineStr">
+        <is>
+          <t>Nusrat Jahan</t>
+        </is>
+      </c>
+      <c r="J276" t="inlineStr">
+        <is>
+          <t>নুসরাত জাহান</t>
+        </is>
+      </c>
+      <c r="K276" t="inlineStr">
+        <is>
+          <t>Mohammed Jafor Iqbal Talukder</t>
+        </is>
+      </c>
+      <c r="L276" t="inlineStr">
+        <is>
+          <t>Saleha Akter</t>
+        </is>
+      </c>
+      <c r="M276" t="inlineStr">
+        <is>
+          <t>CDDL Navy School</t>
+        </is>
+      </c>
+      <c r="N276" t="inlineStr">
+        <is>
+          <t>07</t>
+        </is>
+      </c>
+      <c r="O276" t="inlineStr">
+        <is>
+          <t>03</t>
+        </is>
+      </c>
+      <c r="P276" t="inlineStr">
+        <is>
+          <t>Rubi cement colony,(Rab 7 এর পাশে),North Patenga,Chattogram</t>
+        </is>
+      </c>
+      <c r="Q276" t="inlineStr">
+        <is>
+          <t>01336826867</t>
+        </is>
+      </c>
+      <c r="S276" t="inlineStr">
+        <is>
+          <t>Patenga</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>3849</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>01723088207</t>
+        </is>
+      </c>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>DJF424TGIU</t>
+        </is>
+      </c>
+      <c r="G277" t="inlineStr">
+        <is>
+          <t>2026-10-15 14:29:33</t>
+        </is>
+      </c>
+      <c r="H277" t="inlineStr">
+        <is>
+          <t>Boy</t>
+        </is>
+      </c>
+      <c r="I277" t="inlineStr">
+        <is>
+          <t>Md.Samiul Islam Alvi</t>
+        </is>
+      </c>
+      <c r="J277" t="inlineStr">
+        <is>
+          <t>মো:সামিউল ইসলাম আলভী</t>
+        </is>
+      </c>
+      <c r="K277" t="inlineStr">
+        <is>
+          <t>Md Saiful Islam</t>
+        </is>
+      </c>
+      <c r="L277" t="inlineStr">
+        <is>
+          <t>Sarmeen Akter</t>
+        </is>
+      </c>
+      <c r="M277" t="inlineStr">
+        <is>
+          <t>Ispahani Public School And College</t>
+        </is>
+      </c>
+      <c r="N277" t="inlineStr">
+        <is>
+          <t>09</t>
+        </is>
+      </c>
+      <c r="O277" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="P277" t="inlineStr">
+        <is>
+          <t>Shah Garibullah Housing Society,Road no.1/1,House no.01,Khulshi. Chattogram</t>
+        </is>
+      </c>
+      <c r="Q277" t="inlineStr">
+        <is>
+          <t>01717944271</t>
+        </is>
+      </c>
+      <c r="S277" t="inlineStr">
+        <is>
+          <t>agrabad</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>3850</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>01521735429</t>
+        </is>
+      </c>
+      <c r="D278" t="inlineStr">
+        <is>
+          <t>DJG53FJD7N</t>
+        </is>
+      </c>
+      <c r="G278" t="inlineStr">
+        <is>
+          <t>2026-10-16 10:34:58</t>
+        </is>
+      </c>
+      <c r="H278" t="inlineStr">
+        <is>
+          <t>Girl</t>
+        </is>
+      </c>
+      <c r="I278" t="inlineStr">
+        <is>
+          <t>Tasnia Farin Yusha</t>
+        </is>
+      </c>
+      <c r="J278" t="inlineStr">
+        <is>
+          <t>তাসনিয়া ফারিন ইউশা</t>
+        </is>
+      </c>
+      <c r="K278" t="inlineStr">
+        <is>
+          <t>Mohammad Mojibul Hoque</t>
+        </is>
+      </c>
+      <c r="L278" t="inlineStr">
+        <is>
+          <t>Nilufer Yeasmin</t>
+        </is>
+      </c>
+      <c r="M278" t="inlineStr">
+        <is>
+          <t>Dr. Khastagir Govt. Girls High School</t>
+        </is>
+      </c>
+      <c r="N278" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="O278" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="P278" t="inlineStr">
+        <is>
+          <t>271, Rosulbag C Block, Bakolia, Chattogram</t>
+        </is>
+      </c>
+      <c r="Q278" t="inlineStr">
+        <is>
+          <t>8801970433883</t>
+        </is>
+      </c>
+      <c r="S278" t="inlineStr">
+        <is>
+          <t>dewanhat</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>3852</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>01612938480</t>
+        </is>
+      </c>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>DJG93UQR9T</t>
+        </is>
+      </c>
+      <c r="G279" t="inlineStr">
+        <is>
+          <t>2026-10-16 14:29:51</t>
+        </is>
+      </c>
+      <c r="H279" t="inlineStr">
+        <is>
+          <t>Boy</t>
+        </is>
+      </c>
+      <c r="I279" t="inlineStr">
+        <is>
+          <t>Prantik Barua Dhrubo</t>
+        </is>
+      </c>
+      <c r="J279" t="inlineStr">
+        <is>
+          <t>প্রান্তিক বড়ুয়া ধ্রুব</t>
+        </is>
+      </c>
+      <c r="K279" t="inlineStr">
+        <is>
+          <t>Dipak Barua</t>
+        </is>
+      </c>
+      <c r="L279" t="inlineStr">
+        <is>
+          <t>Priya Barua</t>
+        </is>
+      </c>
+      <c r="M279" t="inlineStr">
+        <is>
+          <t>Green Bell School &amp; College</t>
+        </is>
+      </c>
+      <c r="N279" t="inlineStr">
+        <is>
+          <t>Class Six</t>
+        </is>
+      </c>
+      <c r="O279" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="P279" t="inlineStr">
+        <is>
+          <t>Dhum para Khatgor Pategha Chattagram</t>
+        </is>
+      </c>
+      <c r="Q279" t="inlineStr">
+        <is>
+          <t>01612938480</t>
+        </is>
+      </c>
+      <c r="S279" t="inlineStr">
+        <is>
+          <t>Patenga</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>3853</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>01300480754</t>
+        </is>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>DJG73Z172T</t>
+        </is>
+      </c>
+      <c r="G280" t="inlineStr">
+        <is>
+          <t>2026-10-16 15:29:58</t>
+        </is>
+      </c>
+      <c r="H280" t="inlineStr">
+        <is>
+          <t>Boy</t>
+        </is>
+      </c>
+      <c r="I280" t="inlineStr">
+        <is>
+          <t>MD.Rayhan Alam</t>
+        </is>
+      </c>
+      <c r="J280" t="inlineStr">
+        <is>
+          <t>মোঃ রায়হান আলম</t>
+        </is>
+      </c>
+      <c r="K280" t="inlineStr">
+        <is>
+          <t>Jahangir Alam</t>
+        </is>
+      </c>
+      <c r="L280" t="inlineStr">
+        <is>
+          <t>Rehana Akther</t>
+        </is>
+      </c>
+      <c r="M280" t="inlineStr">
+        <is>
+          <t>Chattogram Collegiate School, Chattogram</t>
+        </is>
+      </c>
+      <c r="N280" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="O280" t="inlineStr">
+        <is>
+          <t>49</t>
+        </is>
+      </c>
+      <c r="P280" t="inlineStr">
+        <is>
+          <t>AK house 121, Chandanpura, Chawk bazar, Chattogram</t>
+        </is>
+      </c>
+      <c r="Q280" t="inlineStr">
+        <is>
+          <t>01851911435</t>
+        </is>
+      </c>
+      <c r="S280" t="inlineStr">
+        <is>
+          <t>dewanhat</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>3854</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>01873029849</t>
+        </is>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>DJG541N0CZ</t>
+        </is>
+      </c>
+      <c r="G281" t="inlineStr">
+        <is>
+          <t>2026-10-16 16:04:01</t>
+        </is>
+      </c>
+      <c r="H281" t="inlineStr">
+        <is>
+          <t>Girl</t>
+        </is>
+      </c>
+      <c r="I281" t="inlineStr">
+        <is>
+          <t>Fahmida khanom alifa</t>
+        </is>
+      </c>
+      <c r="J281" t="inlineStr">
+        <is>
+          <t>ফাহমিদা খানম আলিফা</t>
+        </is>
+      </c>
+      <c r="K281" t="inlineStr">
+        <is>
+          <t>Ayub khan</t>
+        </is>
+      </c>
+      <c r="L281" t="inlineStr">
+        <is>
+          <t>Firoja akther</t>
+        </is>
+      </c>
+      <c r="M281" t="inlineStr">
+        <is>
+          <t>South kattali pran hori model gov't primary school</t>
+        </is>
+      </c>
+      <c r="N281" t="inlineStr">
+        <is>
+          <t>Five</t>
+        </is>
+      </c>
+      <c r="O281" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="P281" t="inlineStr">
+        <is>
+          <t>Sandwip Bhavon,college road,Halishahor, ctg.</t>
+        </is>
+      </c>
+      <c r="Q281" t="inlineStr">
+        <is>
+          <t>01789865054</t>
+        </is>
+      </c>
+      <c r="S281" t="inlineStr">
+        <is>
+          <t>halishahar</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>3856</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>01675271093</t>
+        </is>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>DJG544GCDV</t>
+        </is>
+      </c>
+      <c r="G282" t="inlineStr">
+        <is>
+          <t>2026-10-16 16:59:34</t>
+        </is>
+      </c>
+      <c r="H282" t="inlineStr">
+        <is>
+          <t>Boy</t>
+        </is>
+      </c>
+      <c r="I282" t="inlineStr">
+        <is>
+          <t>Mosaidul Hossain Nihad</t>
+        </is>
+      </c>
+      <c r="J282" t="inlineStr">
+        <is>
+          <t>মোসাইদুল হোসেন নিহাদ</t>
+        </is>
+      </c>
+      <c r="K282" t="inlineStr">
+        <is>
+          <t>Moazzam Hossain Molla</t>
+        </is>
+      </c>
+      <c r="L282" t="inlineStr">
+        <is>
+          <t>Tania Akter</t>
+        </is>
+      </c>
+      <c r="M282" t="inlineStr">
+        <is>
+          <t>Halishahar Cantonment Public School and College</t>
+        </is>
+      </c>
+      <c r="N282" t="inlineStr">
+        <is>
+          <t>Seven</t>
+        </is>
+      </c>
+      <c r="O282" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="P282" t="inlineStr">
+        <is>
+          <t>Lane-2, I-Block, Halishahar, Chattogram</t>
+        </is>
+      </c>
+      <c r="Q282" t="inlineStr">
+        <is>
+          <t>01675271093</t>
+        </is>
+      </c>
+      <c r="S282" t="inlineStr">
+        <is>
+          <t>halishahar</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>3857</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>01723088207</t>
+        </is>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>567</t>
+        </is>
+      </c>
+      <c r="G283" t="inlineStr">
+        <is>
+          <t>2026-10-17 15:50:24</t>
+        </is>
+      </c>
+      <c r="H283" t="inlineStr">
+        <is>
+          <t>Girl</t>
+        </is>
+      </c>
+      <c r="I283" t="inlineStr">
+        <is>
+          <t>Junaira Farisha Islam</t>
+        </is>
+      </c>
+      <c r="J283" t="inlineStr">
+        <is>
+          <t>জুনাইরা ফারিশা ইসলাম</t>
+        </is>
+      </c>
+      <c r="K283" t="inlineStr">
+        <is>
+          <t>Me.Manirul Islam</t>
+        </is>
+      </c>
+      <c r="L283" t="inlineStr">
+        <is>
+          <t>Farhana Akter</t>
+        </is>
+      </c>
+      <c r="M283" t="inlineStr">
+        <is>
+          <t>HCPSC</t>
+        </is>
+      </c>
+      <c r="N283" t="inlineStr">
+        <is>
+          <t>Six</t>
+        </is>
+      </c>
+      <c r="O283" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="P283" t="inlineStr">
+        <is>
+          <t>House #34, Lane#8, Road# 1,Block# A.Halishahar, ctg</t>
+        </is>
+      </c>
+      <c r="Q283" t="inlineStr">
+        <is>
+          <t>01838518567</t>
+        </is>
+      </c>
+      <c r="S283" t="inlineStr">
+        <is>
+          <t>halishahar</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>3858</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>01723088207</t>
+        </is>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>567</t>
+        </is>
+      </c>
+      <c r="G284" t="inlineStr">
+        <is>
+          <t>2026-10-17 15:59:10</t>
+        </is>
+      </c>
+      <c r="H284" t="inlineStr">
+        <is>
+          <t>Boy</t>
+        </is>
+      </c>
+      <c r="I284" t="inlineStr">
+        <is>
+          <t>Zain Riyasat Islam</t>
+        </is>
+      </c>
+      <c r="J284" t="inlineStr">
+        <is>
+          <t>জাইন রিয়াসাত ইসলাম</t>
+        </is>
+      </c>
+      <c r="K284" t="inlineStr">
+        <is>
+          <t>Md.Manirul Islam</t>
+        </is>
+      </c>
+      <c r="L284" t="inlineStr">
+        <is>
+          <t>Farhana Akter</t>
+        </is>
+      </c>
+      <c r="M284" t="inlineStr">
+        <is>
+          <t>HCPSC</t>
+        </is>
+      </c>
+      <c r="N284" t="inlineStr">
+        <is>
+          <t>Four</t>
+        </is>
+      </c>
+      <c r="O284" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="P284" t="inlineStr">
+        <is>
+          <t>House #34, Lane#8, Road# 1,Block# A.Halishahar, ctg</t>
+        </is>
+      </c>
+      <c r="Q284" t="inlineStr">
+        <is>
+          <t>01838518567</t>
+        </is>
+      </c>
+      <c r="S284" t="inlineStr">
+        <is>
+          <t>halishahar</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>3860</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>01836831037</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>DJI469U57W</t>
+        </is>
+      </c>
+      <c r="G285" t="inlineStr">
+        <is>
+          <t>2026-10-18 04:22:09</t>
+        </is>
+      </c>
+      <c r="H285" t="inlineStr">
+        <is>
+          <t>Girl</t>
+        </is>
+      </c>
+      <c r="I285" t="inlineStr">
+        <is>
+          <t>Olin Atfa</t>
+        </is>
+      </c>
+      <c r="J285" t="inlineStr">
+        <is>
+          <t>অলিন আতফা</t>
+        </is>
+      </c>
+      <c r="K285" t="inlineStr">
+        <is>
+          <t>MD. YEASIN ARAFAT</t>
+        </is>
+      </c>
+      <c r="L285" t="inlineStr">
+        <is>
+          <t>SABRIN KHANAM</t>
+        </is>
+      </c>
+      <c r="M285" t="inlineStr">
+        <is>
+          <t>GUL-E-ZAR BEGUM CITY CORP MUSLIM GIRLS HIGH SCHOOL</t>
+        </is>
+      </c>
+      <c r="N285" t="inlineStr">
+        <is>
+          <t>Seven</t>
+        </is>
+      </c>
+      <c r="O285" t="inlineStr">
+        <is>
+          <t>76</t>
+        </is>
+      </c>
+      <c r="P285" t="inlineStr">
+        <is>
+          <t>DC road , chawkbazar, Chittagong</t>
+        </is>
+      </c>
+      <c r="Q285" t="inlineStr">
+        <is>
+          <t>01866358979</t>
+        </is>
+      </c>
+      <c r="S285" t="inlineStr">
+        <is>
+          <t>dewanhat</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>3861</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>01722212464</t>
+        </is>
+      </c>
+      <c r="F286" t="inlineStr">
+        <is>
+          <t>766HHM4N</t>
+        </is>
+      </c>
+      <c r="G286" t="inlineStr">
+        <is>
+          <t>2026-10-20 13:29:09</t>
+        </is>
+      </c>
+      <c r="H286" t="inlineStr">
+        <is>
+          <t>Boy</t>
+        </is>
+      </c>
+      <c r="I286" t="inlineStr">
+        <is>
+          <t>AFSAN NAZRUL AR-RAFI</t>
+        </is>
+      </c>
+      <c r="J286" t="inlineStr">
+        <is>
+          <t>আফসান নজরুল আর-রাফি</t>
+        </is>
+      </c>
+      <c r="K286" t="inlineStr">
+        <is>
+          <t>MD. NAZRUL ISLAM</t>
+        </is>
+      </c>
+      <c r="L286" t="inlineStr">
+        <is>
+          <t>KANICH FATIMA</t>
+        </is>
+      </c>
+      <c r="M286" t="inlineStr">
+        <is>
+          <t>Ispahani Public School &amp; College</t>
+        </is>
+      </c>
+      <c r="N286" t="inlineStr">
+        <is>
+          <t>Five</t>
+        </is>
+      </c>
+      <c r="O286" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
+      <c r="P286" t="inlineStr">
+        <is>
+          <t>Kusumbag R/A, Goribullah shah majar, Khulshi, Chattogram</t>
+        </is>
+      </c>
+      <c r="Q286" t="inlineStr">
+        <is>
+          <t>01953031941</t>
+        </is>
+      </c>
+      <c r="S286" t="inlineStr">
+        <is>
+          <t>dewanhat</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:S271"/>
+  <autoFilter ref="A1:S286"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Use hand-updated rolls/centres for orders 3843-3861 and regenerate their cards
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Admit_Card_Data_2026.xlsx
+++ b/Admit_Card_Data_2026.xlsx
@@ -16159,12 +16159,12 @@
       </c>
       <c r="B271" s="2" t="inlineStr">
         <is>
-          <t>41126048</t>
+          <t>41126040</t>
         </is>
       </c>
       <c r="C271" s="2" t="inlineStr">
         <is>
-          <t>Admit_41126048_Duplicate</t>
+          <t>Admit_41126040_Duplicate</t>
         </is>
       </c>
       <c r="D271" s="2" t="inlineStr">
@@ -16222,12 +16222,12 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>83126042</t>
+          <t>81126057</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>Admit_83126042</t>
+          <t>Admit_81126057</t>
         </is>
       </c>
       <c r="D272" t="inlineStr">
@@ -16265,7 +16265,7 @@
       </c>
       <c r="K272" t="inlineStr">
         <is>
-          <t>সিলভার বেলস কিন্ডারগার্টেন এন্ড গার্লস হাই স্কুল</t>
+          <t>চট্টগ্রাম কলেজিয়েট স্কুল</t>
         </is>
       </c>
       <c r="L272" t="inlineStr">
@@ -16280,12 +16280,12 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>71126054</t>
+          <t>71126059</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>Admit_71126054</t>
+          <t>Admit_71126059</t>
         </is>
       </c>
       <c r="D273" t="inlineStr">
@@ -16338,12 +16338,12 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>51126060</t>
+          <t>51126067</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>Admit_51126060</t>
+          <t>Admit_51126067</t>
         </is>
       </c>
       <c r="D274" t="inlineStr">
@@ -16396,12 +16396,12 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>72226059</t>
+          <t>72226069</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>Admit_72226059</t>
+          <t>Admit_72226069</t>
         </is>
       </c>
       <c r="D275" t="inlineStr">
@@ -16454,12 +16454,12 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>93126020</t>
+          <t>91126020</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>Admit_93126020</t>
+          <t>Admit_91126020</t>
         </is>
       </c>
       <c r="D276" t="inlineStr">
@@ -16497,7 +16497,7 @@
       </c>
       <c r="K276" t="inlineStr">
         <is>
-          <t>সিলভার বেলস কিন্ডারগার্টেন এন্ড গার্লস হাই স্কুল</t>
+          <t>চট্টগ্রাম কলেজিয়েট স্কুল</t>
         </is>
       </c>
       <c r="L276" t="inlineStr">
@@ -16512,12 +16512,12 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>61226058</t>
+          <t>61226065</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>Admit_61226058</t>
+          <t>Admit_61226065</t>
         </is>
       </c>
       <c r="D277" t="inlineStr">
@@ -16570,12 +16570,12 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>62126067</t>
+          <t>62126074</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>Admit_62126067</t>
+          <t>Admit_62126074</t>
         </is>
       </c>
       <c r="D278" t="inlineStr">
@@ -16628,12 +16628,12 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>71126055</t>
+          <t>71126060</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>Admit_71126055</t>
+          <t>Admit_71126060</t>
         </is>
       </c>
       <c r="D279" t="inlineStr">
@@ -16686,12 +16686,12 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>53226123</t>
+          <t>51226084</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>Admit_53226123</t>
+          <t>Admit_51226084</t>
         </is>
       </c>
       <c r="D280" t="inlineStr">
@@ -16729,7 +16729,7 @@
       </c>
       <c r="K280" t="inlineStr">
         <is>
-          <t>সিলভার বেলস কিন্ডারগার্টেন এন্ড গার্লস হাই স্কুল</t>
+          <t>চট্টগ্রাম কলেজিয়েট স্কুল</t>
         </is>
       </c>
       <c r="L280" t="inlineStr">
@@ -16744,12 +16744,12 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>73126050</t>
+          <t>71126061</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>Admit_73126050</t>
+          <t>Admit_71126061</t>
         </is>
       </c>
       <c r="D281" t="inlineStr">
@@ -16787,7 +16787,7 @@
       </c>
       <c r="K281" t="inlineStr">
         <is>
-          <t>সিলভার বেলস কিন্ডারগার্টেন এন্ড গার্লস হাই স্কুল</t>
+          <t>চট্টগ্রাম কলেজিয়েট স্কুল</t>
         </is>
       </c>
       <c r="L281" t="inlineStr">
@@ -16802,12 +16802,12 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>63226077</t>
+          <t>61226066</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>Admit_63226077</t>
+          <t>Admit_61226066</t>
         </is>
       </c>
       <c r="D282" t="inlineStr">
@@ -16845,7 +16845,7 @@
       </c>
       <c r="K282" t="inlineStr">
         <is>
-          <t>সিলভার বেলস কিন্ডারগার্টেন এন্ড গার্লস হাই স্কুল</t>
+          <t>চট্টগ্রাম কলেজিয়েট স্কুল</t>
         </is>
       </c>
       <c r="L282" t="inlineStr">
@@ -16860,12 +16860,12 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>43126087</t>
+          <t>41126054</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>Admit_43126087</t>
+          <t>Admit_41126054</t>
         </is>
       </c>
       <c r="D283" t="inlineStr">
@@ -16903,7 +16903,7 @@
       </c>
       <c r="K283" t="inlineStr">
         <is>
-          <t>সিলভার বেলস কিন্ডারগার্টেন এন্ড গার্লস হাই স্কুল</t>
+          <t>চট্টগ্রাম কলেজিয়েট স্কুল</t>
         </is>
       </c>
       <c r="L283" t="inlineStr">
@@ -16918,12 +16918,12 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>71226068</t>
+          <t>71226070</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>Admit_71226068</t>
+          <t>Admit_71226070</t>
         </is>
       </c>
       <c r="D284" t="inlineStr">
@@ -16976,12 +16976,12 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>51126061</t>
+          <t>51126068</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>Admit_51126061</t>
+          <t>Admit_51126068</t>
         </is>
       </c>
       <c r="D285" t="inlineStr">

</xml_diff>

<commit_message>
Correct student name for roll 51226058 (order 3578) to Sarah Nur Shawli; queue resend
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Admit_Card_Data_2026.xlsx
+++ b/Admit_Card_Data_2026.xlsx
@@ -16,7 +16,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Admit_Data'!$A$1:$M$285</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Separate'!$A$1:$N$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Review'!$A$1:$D$46</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Review'!$A$1:$D$47</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Centre_Map'!$A$1:$C$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Raw_Data'!$A$1:$S$286</definedName>
   </definedNames>
@@ -4501,7 +4501,7 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Hossain Mohiuddin</t>
+          <t>Sarah Nur Shawli</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -17203,7 +17203,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D46"/>
+  <dimension ref="A1:D47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -17356,27 +17356,27 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>3750</v>
+        <v>3578</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Student</t>
+          <t>Name (English)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>MOHAMMED MUHTASIM ISLAM</t>
+          <t>Hossain Mohiuddin</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>same student as order 3506 - kept both, marked in file name</t>
+          <t>name corrected to Sarah Nur Shawli (by user)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>3506</v>
+        <v>3750</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -17390,27 +17390,27 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>same student as order 3750 - kept both, marked in file name</t>
+          <t>same student as order 3506 - kept both, marked in file name</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>3446</v>
+        <v>3506</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Student</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>মোহাম্মদ নুরুল ইসলাম</t>
+          <t>MOHAMMED MUHTASIM ISLAM</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>written in Bangla (kept as entered)</t>
+          <t>same student as order 3750 - kept both, marked in file name</t>
         </is>
       </c>
     </row>
@@ -17420,12 +17420,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>ডাঃ খাস্তগীর সরকারি বালিকা উচ্চ বিদ্যালয়</t>
+          <t>মোহাম্মদ নুরুল ইসলাম</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -17436,7 +17436,7 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>3509</v>
+        <v>3446</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -17445,7 +17445,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>ফুলকি সহজপাঠ বিদ্যালয়</t>
+          <t>ডাঃ খাস্তগীর সরকারি বালিকা উচ্চ বিদ্যালয়</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -17456,16 +17456,16 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>3604</v>
+        <v>3509</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>মোঃ আনোয়ার হোসেন</t>
+          <t>ফুলকি সহজপাঠ বিদ্যালয়</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -17480,12 +17480,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>হালিশহর ক্যান্টনম্যান্ট পাবলিক স্কুল এন্ড কলেজ</t>
+          <t>মোঃ আনোয়ার হোসেন</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -17496,16 +17496,16 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>3639</v>
+        <v>3604</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>মোঃ আবু সায়েম</t>
+          <t>হালিশহর ক্যান্টনম্যান্ট পাবলিক স্কুল এন্ড কলেজ</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -17520,12 +17520,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>বিএএফ শাহীন কলেজ</t>
+          <t>মোঃ আবু সায়েম</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -17536,16 +17536,16 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>3642</v>
+        <v>3639</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>মনির হোসেন</t>
+          <t>বিএএফ শাহীন কলেজ</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -17560,12 +17560,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>বিএএফ শাহীন কলেজ</t>
+          <t>মনির হোসেন</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -17576,16 +17576,16 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>3643</v>
+        <v>3642</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>মো: রেজাউল করিম</t>
+          <t>বিএএফ শাহীন কলেজ</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -17600,12 +17600,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>বিএএফ শাহীন কলেজ</t>
+          <t>মো: রেজাউল করিম</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -17616,16 +17616,16 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>3649</v>
+        <v>3643</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>মোঃ নিজাম উদ্দিন</t>
+          <t>বিএএফ শাহীন কলেজ</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -17640,12 +17640,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>বাংলাদেশ নৌবাহিনী স্কুল এন্ড কলেজ, চট্টগ্রাম</t>
+          <t>মোঃ নিজাম উদ্দিন</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -17656,16 +17656,16 @@
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>3670</v>
+        <v>3649</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>জুলফিকার আলী মিঠু</t>
+          <t>বাংলাদেশ নৌবাহিনী স্কুল এন্ড কলেজ, চট্টগ্রাম</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -17680,12 +17680,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>বিএএফ শাহীন কলেজ</t>
+          <t>জুলফিকার আলী মিঠু</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -17696,7 +17696,7 @@
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>3680</v>
+        <v>3670</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -17705,7 +17705,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>বলুয়ারদীঘি সিটি কর্পোরেশন বালিকা উচ্চ বিদ্যালয়</t>
+          <t>বিএএফ শাহীন কলেজ</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -17716,16 +17716,16 @@
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>3697</v>
+        <v>3680</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>কাকন চক্রবর্তী</t>
+          <t>বলুয়ারদীঘি সিটি কর্পোরেশন বালিকা উচ্চ বিদ্যালয়</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -17740,12 +17740,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>মুসলিম এডুকেশন সোসাইটি উচ্চ বিদ্যালয়</t>
+          <t>কাকন চক্রবর্তী</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -17756,16 +17756,16 @@
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>3718</v>
+        <v>3697</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>মনির আহমদ</t>
+          <t>মুসলিম এডুকেশন সোসাইটি উচ্চ বিদ্যালয়</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -17780,12 +17780,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>হাটহাজারী আনোয়ারুল উলুম নোমানীয়া ফাজিল মাদ্রাসা</t>
+          <t>মনির আহমদ</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -17796,16 +17796,16 @@
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>3724</v>
+        <v>3718</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>মনিরুল হক</t>
+          <t>হাটহাজারী আনোয়ারুল উলুম নোমানীয়া ফাজিল মাদ্রাসা</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -17820,12 +17820,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>বাহমনিখীল সরকারি প্রাথমিক বিদ্যালয়</t>
+          <t>মনিরুল হক</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -17836,16 +17836,16 @@
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>3748</v>
+        <v>3724</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>আবু বক্কর সিদ্দিক</t>
+          <t>বাহমনিখীল সরকারি প্রাথমিক বিদ্যালয়</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -17860,12 +17860,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>হালিশহর ক্যান্টনমেন্ট পাবলিক স্কুল এন্ড কলেজ</t>
+          <t>আবু বক্কর সিদ্দিক</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -17876,16 +17876,16 @@
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>3770</v>
+        <v>3748</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>মোহাম্মদ রেজাউল করিম</t>
+          <t>হালিশহর ক্যান্টনমেন্ট পাবলিক স্কুল এন্ড কলেজ</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -17900,12 +17900,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>রেলওয়ে পাবলিক স্কুল এন্ড কলেজ</t>
+          <t>মোহাম্মদ রেজাউল করিম</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -17916,16 +17916,16 @@
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>3773</v>
+        <v>3770</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>মোহাম্মদ রেজাউল করিম</t>
+          <t>রেলওয়ে পাবলিক স্কুল এন্ড কলেজ</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -17940,12 +17940,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>সেন্ট্রাল পাবলিক স্কুল এন্ড কলেজ</t>
+          <t>মোহাম্মদ রেজাউল করিম</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -17956,16 +17956,16 @@
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>3796</v>
+        <v>3773</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>মোহাম্মদ নওশাদ ইকবাল</t>
+          <t>সেন্ট্রাল পাবলিক স্কুল এন্ড কলেজ</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -17980,12 +17980,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>ইস্পাহানি পাবলিক স্কুল এন্ড কলেজ, চট্টগ্রাম।</t>
+          <t>মোহাম্মদ নওশাদ ইকবাল</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -17996,16 +17996,16 @@
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>3797</v>
+        <v>3796</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>মোহাম্মদ নওশাদ ইকবাল</t>
+          <t>ইস্পাহানি পাবলিক স্কুল এন্ড কলেজ, চট্টগ্রাম।</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -18020,12 +18020,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>ইস্পাহানি পাবলিক স্কুল এন্ড কলেজ, চট্টগ্রাম।</t>
+          <t>মোহাম্মদ নওশাদ ইকবাল</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -18036,16 +18036,16 @@
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>3835</v>
+        <v>3797</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>মো ইউসুফ</t>
+          <t>ইস্পাহানি পাবলিক স্কুল এন্ড কলেজ, চট্টগ্রাম।</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -18060,12 +18060,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>সি এম পি স্কুল এন্ড কলেজ</t>
+          <t>মো ইউসুফ</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -18076,16 +18076,16 @@
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>3840</v>
+        <v>3835</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>শাহা জাহান</t>
+          <t>সি এম পি স্কুল এন্ড কলেজ</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -18100,12 +18100,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>বাকলিয়া আদর্শ বালিকা উচ্চ বিদ্যালয়</t>
+          <t>শাহা জাহান</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -18116,26 +18116,46 @@
     </row>
     <row r="46">
       <c r="A46" t="n">
+        <v>3840</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Name of School</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>বাকলিয়া আদর্শ বালিকা উচ্চ বিদ্যালয়</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>written in Bangla (kept as entered)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
         <v>3846</v>
       </c>
-      <c r="B46" t="inlineStr">
+      <c r="B47" t="inlineStr">
         <is>
           <t>Name of School</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="C47" t="inlineStr">
         <is>
           <t>মোঃ আরিফুল ইসলাম</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr">
+      <c r="D47" t="inlineStr">
         <is>
           <t>written in Bangla (kept as entered)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D46"/>
+  <autoFilter ref="A1:D47"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Correct school for roll 53126056 (order 3507); queue resend
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Admit_Card_Data_2026.xlsx
+++ b/Admit_Card_Data_2026.xlsx
@@ -16,7 +16,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Admit_Data'!$A$1:$M$285</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Separate'!$A$1:$N$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Review'!$A$1:$D$47</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Review'!$A$1:$D$48</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Centre_Map'!$A$1:$C$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Raw_Data'!$A$1:$S$286</definedName>
   </definedNames>
@@ -968,7 +968,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Mohiuddin Rasel</t>
+          <t>Uttar Kattali Alhaz Mostofa Hakim High School</t>
         </is>
       </c>
       <c r="H9" t="n">
@@ -17203,7 +17203,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D47"/>
+  <dimension ref="A1:D48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -17416,21 +17416,21 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>3446</v>
+        <v>3507</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>মোহাম্মদ নুরুল ইসলাম</t>
+          <t>Mohiuddin Rasel</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>written in Bangla (kept as entered)</t>
+          <t>school corrected to Uttar Kattali Alhaz Mostofa Hakim High School (by user)</t>
         </is>
       </c>
     </row>
@@ -17440,12 +17440,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>ডাঃ খাস্তগীর সরকারি বালিকা উচ্চ বিদ্যালয়</t>
+          <t>মোহাম্মদ নুরুল ইসলাম</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -17456,7 +17456,7 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>3509</v>
+        <v>3446</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -17465,7 +17465,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>ফুলকি সহজপাঠ বিদ্যালয়</t>
+          <t>ডাঃ খাস্তগীর সরকারি বালিকা উচ্চ বিদ্যালয়</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -17476,16 +17476,16 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>3604</v>
+        <v>3509</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>মোঃ আনোয়ার হোসেন</t>
+          <t>ফুলকি সহজপাঠ বিদ্যালয়</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -17500,12 +17500,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>হালিশহর ক্যান্টনম্যান্ট পাবলিক স্কুল এন্ড কলেজ</t>
+          <t>মোঃ আনোয়ার হোসেন</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -17516,16 +17516,16 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>3639</v>
+        <v>3604</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>মোঃ আবু সায়েম</t>
+          <t>হালিশহর ক্যান্টনম্যান্ট পাবলিক স্কুল এন্ড কলেজ</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -17540,12 +17540,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>বিএএফ শাহীন কলেজ</t>
+          <t>মোঃ আবু সায়েম</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -17556,16 +17556,16 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>3642</v>
+        <v>3639</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>মনির হোসেন</t>
+          <t>বিএএফ শাহীন কলেজ</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -17580,12 +17580,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>বিএএফ শাহীন কলেজ</t>
+          <t>মনির হোসেন</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -17596,16 +17596,16 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>3643</v>
+        <v>3642</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>মো: রেজাউল করিম</t>
+          <t>বিএএফ শাহীন কলেজ</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -17620,12 +17620,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>বিএএফ শাহীন কলেজ</t>
+          <t>মো: রেজাউল করিম</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -17636,16 +17636,16 @@
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>3649</v>
+        <v>3643</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>মোঃ নিজাম উদ্দিন</t>
+          <t>বিএএফ শাহীন কলেজ</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -17660,12 +17660,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>বাংলাদেশ নৌবাহিনী স্কুল এন্ড কলেজ, চট্টগ্রাম</t>
+          <t>মোঃ নিজাম উদ্দিন</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -17676,16 +17676,16 @@
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>3670</v>
+        <v>3649</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>জুলফিকার আলী মিঠু</t>
+          <t>বাংলাদেশ নৌবাহিনী স্কুল এন্ড কলেজ, চট্টগ্রাম</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -17700,12 +17700,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>বিএএফ শাহীন কলেজ</t>
+          <t>জুলফিকার আলী মিঠু</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -17716,7 +17716,7 @@
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>3680</v>
+        <v>3670</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -17725,7 +17725,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>বলুয়ারদীঘি সিটি কর্পোরেশন বালিকা উচ্চ বিদ্যালয়</t>
+          <t>বিএএফ শাহীন কলেজ</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -17736,16 +17736,16 @@
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>3697</v>
+        <v>3680</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>কাকন চক্রবর্তী</t>
+          <t>বলুয়ারদীঘি সিটি কর্পোরেশন বালিকা উচ্চ বিদ্যালয়</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -17760,12 +17760,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>মুসলিম এডুকেশন সোসাইটি উচ্চ বিদ্যালয়</t>
+          <t>কাকন চক্রবর্তী</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -17776,16 +17776,16 @@
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>3718</v>
+        <v>3697</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>মনির আহমদ</t>
+          <t>মুসলিম এডুকেশন সোসাইটি উচ্চ বিদ্যালয়</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -17800,12 +17800,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>হাটহাজারী আনোয়ারুল উলুম নোমানীয়া ফাজিল মাদ্রাসা</t>
+          <t>মনির আহমদ</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -17816,16 +17816,16 @@
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>3724</v>
+        <v>3718</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>মনিরুল হক</t>
+          <t>হাটহাজারী আনোয়ারুল উলুম নোমানীয়া ফাজিল মাদ্রাসা</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -17840,12 +17840,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>বাহমনিখীল সরকারি প্রাথমিক বিদ্যালয়</t>
+          <t>মনিরুল হক</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -17856,16 +17856,16 @@
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>3748</v>
+        <v>3724</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>আবু বক্কর সিদ্দিক</t>
+          <t>বাহমনিখীল সরকারি প্রাথমিক বিদ্যালয়</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -17880,12 +17880,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>হালিশহর ক্যান্টনমেন্ট পাবলিক স্কুল এন্ড কলেজ</t>
+          <t>আবু বক্কর সিদ্দিক</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -17896,16 +17896,16 @@
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>3770</v>
+        <v>3748</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>মোহাম্মদ রেজাউল করিম</t>
+          <t>হালিশহর ক্যান্টনমেন্ট পাবলিক স্কুল এন্ড কলেজ</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -17920,12 +17920,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>রেলওয়ে পাবলিক স্কুল এন্ড কলেজ</t>
+          <t>মোহাম্মদ রেজাউল করিম</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -17936,16 +17936,16 @@
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>3773</v>
+        <v>3770</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>মোহাম্মদ রেজাউল করিম</t>
+          <t>রেলওয়ে পাবলিক স্কুল এন্ড কলেজ</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -17960,12 +17960,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>সেন্ট্রাল পাবলিক স্কুল এন্ড কলেজ</t>
+          <t>মোহাম্মদ রেজাউল করিম</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -17976,16 +17976,16 @@
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>3796</v>
+        <v>3773</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>মোহাম্মদ নওশাদ ইকবাল</t>
+          <t>সেন্ট্রাল পাবলিক স্কুল এন্ড কলেজ</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -18000,12 +18000,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>ইস্পাহানি পাবলিক স্কুল এন্ড কলেজ, চট্টগ্রাম।</t>
+          <t>মোহাম্মদ নওশাদ ইকবাল</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -18016,16 +18016,16 @@
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>3797</v>
+        <v>3796</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>মোহাম্মদ নওশাদ ইকবাল</t>
+          <t>ইস্পাহানি পাবলিক স্কুল এন্ড কলেজ, চট্টগ্রাম।</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -18040,12 +18040,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>ইস্পাহানি পাবলিক স্কুল এন্ড কলেজ, চট্টগ্রাম।</t>
+          <t>মোহাম্মদ নওশাদ ইকবাল</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -18056,16 +18056,16 @@
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>3835</v>
+        <v>3797</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>মো ইউসুফ</t>
+          <t>ইস্পাহানি পাবলিক স্কুল এন্ড কলেজ, চট্টগ্রাম।</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -18080,12 +18080,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>সি এম পি স্কুল এন্ড কলেজ</t>
+          <t>মো ইউসুফ</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -18096,16 +18096,16 @@
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>3840</v>
+        <v>3835</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>শাহা জাহান</t>
+          <t>সি এম পি স্কুল এন্ড কলেজ</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -18120,12 +18120,12 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>বাকলিয়া আদর্শ বালিকা উচ্চ বিদ্যালয়</t>
+          <t>শাহা জাহান</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -18136,26 +18136,46 @@
     </row>
     <row r="47">
       <c r="A47" t="n">
+        <v>3840</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Name of School</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>বাকলিয়া আদর্শ বালিকা উচ্চ বিদ্যালয়</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>written in Bangla (kept as entered)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
         <v>3846</v>
       </c>
-      <c r="B47" t="inlineStr">
+      <c r="B48" t="inlineStr">
         <is>
           <t>Name of School</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
+      <c r="C48" t="inlineStr">
         <is>
           <t>মোঃ আরিফুল ইসলাম</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
+      <c r="D48" t="inlineStr">
         <is>
           <t>written in Bangla (kept as entered)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D47"/>
+  <autoFilter ref="A1:D48"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Correct school for roll 71126059 (order 3846); queue resend
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Admit_Card_Data_2026.xlsx
+++ b/Admit_Card_Data_2026.xlsx
@@ -16,7 +16,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Admit_Data'!$A$1:$M$285</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Separate'!$A$1:$N$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Review'!$A$1:$D$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Review'!$A$1:$D$49</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Centre_Map'!$A$1:$C$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Raw_Data'!$A$1:$S$286</definedName>
   </definedNames>
@@ -16305,7 +16305,7 @@
       </c>
       <c r="G273" t="inlineStr">
         <is>
-          <t>মোঃ আরিফুল ইসলাম</t>
+          <t>Chattogram Collegiate School</t>
         </is>
       </c>
       <c r="H273" t="n">
@@ -17203,7 +17203,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D48"/>
+  <dimension ref="A1:D49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -17416,7 +17416,7 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>3507</v>
+        <v>3846</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -17425,32 +17425,32 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Mohiuddin Rasel</t>
+          <t>মোঃ আরিফুল ইসলাম</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>school corrected to Uttar Kattali Alhaz Mostofa Hakim High School (by user)</t>
+          <t>school corrected to Chattogram Collegiate School (by user)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>3446</v>
+        <v>3507</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>মোহাম্মদ নুরুল ইসলাম</t>
+          <t>Mohiuddin Rasel</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>written in Bangla (kept as entered)</t>
+          <t>school corrected to Uttar Kattali Alhaz Mostofa Hakim High School (by user)</t>
         </is>
       </c>
     </row>
@@ -17460,12 +17460,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>ডাঃ খাস্তগীর সরকারি বালিকা উচ্চ বিদ্যালয়</t>
+          <t>মোহাম্মদ নুরুল ইসলাম</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -17476,7 +17476,7 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>3509</v>
+        <v>3446</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -17485,7 +17485,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>ফুলকি সহজপাঠ বিদ্যালয়</t>
+          <t>ডাঃ খাস্তগীর সরকারি বালিকা উচ্চ বিদ্যালয়</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -17496,16 +17496,16 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>3604</v>
+        <v>3509</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>মোঃ আনোয়ার হোসেন</t>
+          <t>ফুলকি সহজপাঠ বিদ্যালয়</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -17520,12 +17520,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>হালিশহর ক্যান্টনম্যান্ট পাবলিক স্কুল এন্ড কলেজ</t>
+          <t>মোঃ আনোয়ার হোসেন</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -17536,16 +17536,16 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>3639</v>
+        <v>3604</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>মোঃ আবু সায়েম</t>
+          <t>হালিশহর ক্যান্টনম্যান্ট পাবলিক স্কুল এন্ড কলেজ</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -17560,12 +17560,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>বিএএফ শাহীন কলেজ</t>
+          <t>মোঃ আবু সায়েম</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -17576,16 +17576,16 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>3642</v>
+        <v>3639</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>মনির হোসেন</t>
+          <t>বিএএফ শাহীন কলেজ</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -17600,12 +17600,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>বিএএফ শাহীন কলেজ</t>
+          <t>মনির হোসেন</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -17616,16 +17616,16 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>3643</v>
+        <v>3642</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>মো: রেজাউল করিম</t>
+          <t>বিএএফ শাহীন কলেজ</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -17640,12 +17640,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>বিএএফ শাহীন কলেজ</t>
+          <t>মো: রেজাউল করিম</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -17656,16 +17656,16 @@
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>3649</v>
+        <v>3643</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>মোঃ নিজাম উদ্দিন</t>
+          <t>বিএএফ শাহীন কলেজ</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -17680,12 +17680,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>বাংলাদেশ নৌবাহিনী স্কুল এন্ড কলেজ, চট্টগ্রাম</t>
+          <t>মোঃ নিজাম উদ্দিন</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -17696,16 +17696,16 @@
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>3670</v>
+        <v>3649</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>জুলফিকার আলী মিঠু</t>
+          <t>বাংলাদেশ নৌবাহিনী স্কুল এন্ড কলেজ, চট্টগ্রাম</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -17720,12 +17720,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>বিএএফ শাহীন কলেজ</t>
+          <t>জুলফিকার আলী মিঠু</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -17736,7 +17736,7 @@
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>3680</v>
+        <v>3670</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -17745,7 +17745,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>বলুয়ারদীঘি সিটি কর্পোরেশন বালিকা উচ্চ বিদ্যালয়</t>
+          <t>বিএএফ শাহীন কলেজ</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -17756,16 +17756,16 @@
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>3697</v>
+        <v>3680</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>কাকন চক্রবর্তী</t>
+          <t>বলুয়ারদীঘি সিটি কর্পোরেশন বালিকা উচ্চ বিদ্যালয়</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -17780,12 +17780,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>মুসলিম এডুকেশন সোসাইটি উচ্চ বিদ্যালয়</t>
+          <t>কাকন চক্রবর্তী</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -17796,16 +17796,16 @@
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>3718</v>
+        <v>3697</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>মনির আহমদ</t>
+          <t>মুসলিম এডুকেশন সোসাইটি উচ্চ বিদ্যালয়</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -17820,12 +17820,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>হাটহাজারী আনোয়ারুল উলুম নোমানীয়া ফাজিল মাদ্রাসা</t>
+          <t>মনির আহমদ</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -17836,16 +17836,16 @@
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>3724</v>
+        <v>3718</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>মনিরুল হক</t>
+          <t>হাটহাজারী আনোয়ারুল উলুম নোমানীয়া ফাজিল মাদ্রাসা</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -17860,12 +17860,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>বাহমনিখীল সরকারি প্রাথমিক বিদ্যালয়</t>
+          <t>মনিরুল হক</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -17876,16 +17876,16 @@
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>3748</v>
+        <v>3724</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>আবু বক্কর সিদ্দিক</t>
+          <t>বাহমনিখীল সরকারি প্রাথমিক বিদ্যালয়</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -17900,12 +17900,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>হালিশহর ক্যান্টনমেন্ট পাবলিক স্কুল এন্ড কলেজ</t>
+          <t>আবু বক্কর সিদ্দিক</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -17916,16 +17916,16 @@
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>3770</v>
+        <v>3748</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>মোহাম্মদ রেজাউল করিম</t>
+          <t>হালিশহর ক্যান্টনমেন্ট পাবলিক স্কুল এন্ড কলেজ</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -17940,12 +17940,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>রেলওয়ে পাবলিক স্কুল এন্ড কলেজ</t>
+          <t>মোহাম্মদ রেজাউল করিম</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -17956,16 +17956,16 @@
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>3773</v>
+        <v>3770</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>মোহাম্মদ রেজাউল করিম</t>
+          <t>রেলওয়ে পাবলিক স্কুল এন্ড কলেজ</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -17980,12 +17980,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>সেন্ট্রাল পাবলিক স্কুল এন্ড কলেজ</t>
+          <t>মোহাম্মদ রেজাউল করিম</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -17996,16 +17996,16 @@
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>3796</v>
+        <v>3773</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>মোহাম্মদ নওশাদ ইকবাল</t>
+          <t>সেন্ট্রাল পাবলিক স্কুল এন্ড কলেজ</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -18020,12 +18020,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>ইস্পাহানি পাবলিক স্কুল এন্ড কলেজ, চট্টগ্রাম।</t>
+          <t>মোহাম্মদ নওশাদ ইকবাল</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -18036,16 +18036,16 @@
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>3797</v>
+        <v>3796</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>মোহাম্মদ নওশাদ ইকবাল</t>
+          <t>ইস্পাহানি পাবলিক স্কুল এন্ড কলেজ, চট্টগ্রাম।</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -18060,12 +18060,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>ইস্পাহানি পাবলিক স্কুল এন্ড কলেজ, চট্টগ্রাম।</t>
+          <t>মোহাম্মদ নওশাদ ইকবাল</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -18076,16 +18076,16 @@
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>3835</v>
+        <v>3797</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>মো ইউসুফ</t>
+          <t>ইস্পাহানি পাবলিক স্কুল এন্ড কলেজ, চট্টগ্রাম।</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -18100,12 +18100,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>সি এম পি স্কুল এন্ড কলেজ</t>
+          <t>মো ইউসুফ</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -18116,16 +18116,16 @@
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>3840</v>
+        <v>3835</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>শাহা জাহান</t>
+          <t>সি এম পি স্কুল এন্ড কলেজ</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -18140,12 +18140,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>বাকলিয়া আদর্শ বালিকা উচ্চ বিদ্যালয়</t>
+          <t>শাহা জাহান</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -18156,26 +18156,46 @@
     </row>
     <row r="48">
       <c r="A48" t="n">
+        <v>3840</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Name of School</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>বাকলিয়া আদর্শ বালিকা উচ্চ বিদ্যালয়</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>written in Bangla (kept as entered)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
         <v>3846</v>
       </c>
-      <c r="B48" t="inlineStr">
+      <c r="B49" t="inlineStr">
         <is>
           <t>Name of School</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr">
+      <c r="C49" t="inlineStr">
         <is>
           <t>মোঃ আরিফুল ইসলাম</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr">
+      <c r="D49" t="inlineStr">
         <is>
           <t>written in Bangla (kept as entered)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D48"/>
+  <autoFilter ref="A1:D49"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Correct student name for 41226063 (order 3795) and father's name for 71226067 (order 3841); queue resends
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Admit_Card_Data_2026.xlsx
+++ b/Admit_Card_Data_2026.xlsx
@@ -16,7 +16,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Admit_Data'!$A$1:$M$285</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Separate'!$A$1:$N$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Review'!$A$1:$D$49</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Review'!$A$1:$D$51</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Centre_Map'!$A$1:$C$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Raw_Data'!$A$1:$S$286</definedName>
   </definedNames>
@@ -14898,7 +14898,7 @@
       </c>
       <c r="E249" t="inlineStr">
         <is>
-          <t>M. Jahirul Islam</t>
+          <t>Miskatul Jannat Labiba</t>
         </is>
       </c>
       <c r="F249" t="inlineStr">
@@ -16063,7 +16063,7 @@
       </c>
       <c r="F269" t="inlineStr">
         <is>
-          <t>Md Absul mannan vhyain</t>
+          <t>Md Abdul mannan vhyain</t>
         </is>
       </c>
       <c r="G269" t="inlineStr">
@@ -17203,7 +17203,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D49"/>
+  <dimension ref="A1:D51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -17276,27 +17276,27 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>3600</v>
+        <v>3841</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Mobile (Online)</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>0183519086</t>
+          <t>Md Absul mannan vhyain</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>invalid mobile (10 digits); replaced with Bkash number +8801835190860</t>
+          <t>father's name corrected to Md Abdul mannan vhyain (by user)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>3534</v>
+        <v>3600</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -17305,18 +17305,18 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>101812378354</t>
+          <t>0183519086</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>invalid mobile (12 digits); replaced with Bkash number +8801812378354</t>
+          <t>invalid mobile (10 digits); replaced with Bkash number +8801835190860</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>3648</v>
+        <v>3534</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -17325,158 +17325,158 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>017418691933</t>
+          <t>101812378354</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>invalid mobile (12 digits); replaced with Nagad Number +8801819315767 - different number, please confirm</t>
+          <t>invalid mobile (12 digits); replaced with Bkash number +8801812378354</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>3843</v>
+        <v>3648</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Student</t>
+          <t>Mobile (Online)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Safwan Zaman Ahnaf</t>
+          <t>017418691933</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>likely same student as order 3561 - kept, marked in file name</t>
+          <t>invalid mobile (12 digits); replaced with Nagad Number +8801819315767 - different number, please confirm</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>3578</v>
+        <v>3843</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Name (English)</t>
+          <t>Student</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Hossain Mohiuddin</t>
+          <t>Safwan Zaman Ahnaf</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>name corrected to Sarah Nur Shawli (by user)</t>
+          <t>likely same student as order 3561 - kept, marked in file name</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>3750</v>
+        <v>3795</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Student</t>
+          <t>Name (English)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>MOHAMMED MUHTASIM ISLAM</t>
+          <t>M. Jahirul Islam</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>same student as order 3506 - kept both, marked in file name</t>
+          <t>name corrected to Miskatul Jannat Labiba (by user)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>3506</v>
+        <v>3578</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Student</t>
+          <t>Name (English)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>MOHAMMED MUHTASIM ISLAM</t>
+          <t>Hossain Mohiuddin</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>same student as order 3750 - kept both, marked in file name</t>
+          <t>name corrected to Sarah Nur Shawli (by user)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>3846</v>
+        <v>3750</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Student</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>মোঃ আরিফুল ইসলাম</t>
+          <t>MOHAMMED MUHTASIM ISLAM</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>school corrected to Chattogram Collegiate School (by user)</t>
+          <t>same student as order 3506 - kept both, marked in file name</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>3507</v>
+        <v>3506</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Student</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Mohiuddin Rasel</t>
+          <t>MOHAMMED MUHTASIM ISLAM</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>school corrected to Uttar Kattali Alhaz Mostofa Hakim High School (by user)</t>
+          <t>same student as order 3750 - kept both, marked in file name</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>3446</v>
+        <v>3846</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>মোহাম্মদ নুরুল ইসলাম</t>
+          <t>মোঃ আরিফুল ইসলাম</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>written in Bangla (kept as entered)</t>
+          <t>school corrected to Chattogram Collegiate School (by user)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>3446</v>
+        <v>3507</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -17485,27 +17485,27 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>ডাঃ খাস্তগীর সরকারি বালিকা উচ্চ বিদ্যালয়</t>
+          <t>Mohiuddin Rasel</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>written in Bangla (kept as entered)</t>
+          <t>school corrected to Uttar Kattali Alhaz Mostofa Hakim High School (by user)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>3509</v>
+        <v>3446</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>ফুলকি সহজপাঠ বিদ্যালয়</t>
+          <t>মোহাম্মদ নুরুল ইসলাম</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -17516,16 +17516,16 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>3604</v>
+        <v>3446</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>মোঃ আনোয়ার হোসেন</t>
+          <t>ডাঃ খাস্তগীর সরকারি বালিকা উচ্চ বিদ্যালয়</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -17536,7 +17536,7 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>3604</v>
+        <v>3509</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -17545,7 +17545,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>হালিশহর ক্যান্টনম্যান্ট পাবলিক স্কুল এন্ড কলেজ</t>
+          <t>ফুলকি সহজপাঠ বিদ্যালয়</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -17556,7 +17556,7 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>3639</v>
+        <v>3604</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -17565,7 +17565,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>মোঃ আবু সায়েম</t>
+          <t>মোঃ আনোয়ার হোসেন</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -17576,7 +17576,7 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>3639</v>
+        <v>3604</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -17585,7 +17585,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>বিএএফ শাহীন কলেজ</t>
+          <t>হালিশহর ক্যান্টনম্যান্ট পাবলিক স্কুল এন্ড কলেজ</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -17596,7 +17596,7 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>3642</v>
+        <v>3639</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -17605,7 +17605,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>মনির হোসেন</t>
+          <t>মোঃ আবু সায়েম</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -17616,7 +17616,7 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>3642</v>
+        <v>3639</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -17636,7 +17636,7 @@
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>3643</v>
+        <v>3642</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -17645,7 +17645,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>মো: রেজাউল করিম</t>
+          <t>মনির হোসেন</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -17656,7 +17656,7 @@
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>3643</v>
+        <v>3642</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -17676,7 +17676,7 @@
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>3649</v>
+        <v>3643</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -17685,7 +17685,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>মোঃ নিজাম উদ্দিন</t>
+          <t>মো: রেজাউল করিম</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -17696,7 +17696,7 @@
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>3649</v>
+        <v>3643</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -17705,7 +17705,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>বাংলাদেশ নৌবাহিনী স্কুল এন্ড কলেজ, চট্টগ্রাম</t>
+          <t>বিএএফ শাহীন কলেজ</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -17716,7 +17716,7 @@
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>3670</v>
+        <v>3649</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -17725,7 +17725,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>জুলফিকার আলী মিঠু</t>
+          <t>মোঃ নিজাম উদ্দিন</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -17736,7 +17736,7 @@
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>3670</v>
+        <v>3649</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -17745,7 +17745,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>বিএএফ শাহীন কলেজ</t>
+          <t>বাংলাদেশ নৌবাহিনী স্কুল এন্ড কলেজ, চট্টগ্রাম</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -17756,16 +17756,16 @@
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>3680</v>
+        <v>3670</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>বলুয়ারদীঘি সিটি কর্পোরেশন বালিকা উচ্চ বিদ্যালয়</t>
+          <t>জুলফিকার আলী মিঠু</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -17776,16 +17776,16 @@
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>3697</v>
+        <v>3670</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>কাকন চক্রবর্তী</t>
+          <t>বিএএফ শাহীন কলেজ</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -17796,7 +17796,7 @@
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>3697</v>
+        <v>3680</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -17805,7 +17805,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>মুসলিম এডুকেশন সোসাইটি উচ্চ বিদ্যালয়</t>
+          <t>বলুয়ারদীঘি সিটি কর্পোরেশন বালিকা উচ্চ বিদ্যালয়</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -17816,7 +17816,7 @@
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>3718</v>
+        <v>3697</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -17825,7 +17825,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>মনির আহমদ</t>
+          <t>কাকন চক্রবর্তী</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -17836,7 +17836,7 @@
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>3718</v>
+        <v>3697</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -17845,7 +17845,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>হাটহাজারী আনোয়ারুল উলুম নোমানীয়া ফাজিল মাদ্রাসা</t>
+          <t>মুসলিম এডুকেশন সোসাইটি উচ্চ বিদ্যালয়</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -17856,7 +17856,7 @@
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>3724</v>
+        <v>3718</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -17865,7 +17865,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>মনিরুল হক</t>
+          <t>মনির আহমদ</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -17876,7 +17876,7 @@
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>3724</v>
+        <v>3718</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -17885,7 +17885,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>বাহমনিখীল সরকারি প্রাথমিক বিদ্যালয়</t>
+          <t>হাটহাজারী আনোয়ারুল উলুম নোমানীয়া ফাজিল মাদ্রাসা</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -17896,7 +17896,7 @@
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>3748</v>
+        <v>3724</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -17905,7 +17905,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>আবু বক্কর সিদ্দিক</t>
+          <t>মনিরুল হক</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -17916,7 +17916,7 @@
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>3748</v>
+        <v>3724</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -17925,7 +17925,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>হালিশহর ক্যান্টনমেন্ট পাবলিক স্কুল এন্ড কলেজ</t>
+          <t>বাহমনিখীল সরকারি প্রাথমিক বিদ্যালয়</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -17936,7 +17936,7 @@
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>3770</v>
+        <v>3748</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -17945,7 +17945,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>মোহাম্মদ রেজাউল করিম</t>
+          <t>আবু বক্কর সিদ্দিক</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -17956,7 +17956,7 @@
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>3770</v>
+        <v>3748</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -17965,7 +17965,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>রেলওয়ে পাবলিক স্কুল এন্ড কলেজ</t>
+          <t>হালিশহর ক্যান্টনমেন্ট পাবলিক স্কুল এন্ড কলেজ</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -17976,7 +17976,7 @@
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>3773</v>
+        <v>3770</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -17996,7 +17996,7 @@
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>3773</v>
+        <v>3770</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -18005,7 +18005,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>সেন্ট্রাল পাবলিক স্কুল এন্ড কলেজ</t>
+          <t>রেলওয়ে পাবলিক স্কুল এন্ড কলেজ</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -18016,7 +18016,7 @@
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>3796</v>
+        <v>3773</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -18025,7 +18025,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>মোহাম্মদ নওশাদ ইকবাল</t>
+          <t>মোহাম্মদ রেজাউল করিম</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -18036,7 +18036,7 @@
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>3796</v>
+        <v>3773</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -18045,7 +18045,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>ইস্পাহানি পাবলিক স্কুল এন্ড কলেজ, চট্টগ্রাম।</t>
+          <t>সেন্ট্রাল পাবলিক স্কুল এন্ড কলেজ</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -18056,7 +18056,7 @@
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>3797</v>
+        <v>3796</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -18076,7 +18076,7 @@
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>3797</v>
+        <v>3796</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -18096,7 +18096,7 @@
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>3835</v>
+        <v>3797</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
@@ -18105,7 +18105,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>মো ইউসুফ</t>
+          <t>মোহাম্মদ নওশাদ ইকবাল</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -18116,7 +18116,7 @@
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>3835</v>
+        <v>3797</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
@@ -18125,7 +18125,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>সি এম পি স্কুল এন্ড কলেজ</t>
+          <t>ইস্পাহানি পাবলিক স্কুল এন্ড কলেজ, চট্টগ্রাম।</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -18136,7 +18136,7 @@
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>3840</v>
+        <v>3835</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
@@ -18145,7 +18145,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>শাহা জাহান</t>
+          <t>মো ইউসুফ</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -18156,7 +18156,7 @@
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>3840</v>
+        <v>3835</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
@@ -18165,7 +18165,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>বাকলিয়া আদর্শ বালিকা উচ্চ বিদ্যালয়</t>
+          <t>সি এম পি স্কুল এন্ড কলেজ</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -18176,26 +18176,66 @@
     </row>
     <row r="49">
       <c r="A49" t="n">
+        <v>3840</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Fathers Name</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>শাহা জাহান</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>written in Bangla (kept as entered)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>3840</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Name of School</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>বাকলিয়া আদর্শ বালিকা উচ্চ বিদ্যালয়</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>written in Bangla (kept as entered)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
         <v>3846</v>
       </c>
-      <c r="B49" t="inlineStr">
+      <c r="B51" t="inlineStr">
         <is>
           <t>Name of School</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
+      <c r="C51" t="inlineStr">
         <is>
           <t>মোঃ আরিফুল ইসলাম</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr">
+      <c r="D51" t="inlineStr">
         <is>
           <t>written in Bangla (kept as entered)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D49"/>
+  <autoFilter ref="A1:D51"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Correct school for roll 11126020 (order 3667); queue resend
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Admit_Card_Data_2026.xlsx
+++ b/Admit_Card_Data_2026.xlsx
@@ -16,7 +16,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Admit_Data'!$A$1:$M$285</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Separate'!$A$1:$N$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Review'!$A$1:$D$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Review'!$A$1:$D$52</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Centre_Map'!$A$1:$C$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Raw_Data'!$A$1:$S$286</definedName>
   </definedNames>
@@ -8987,7 +8987,7 @@
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>Nazmin Akter</t>
+          <t>Railway public High School</t>
         </is>
       </c>
       <c r="H147" t="n">
@@ -17203,7 +17203,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D51"/>
+  <dimension ref="A1:D52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -17476,7 +17476,7 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>3507</v>
+        <v>3667</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -17485,32 +17485,32 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Mohiuddin Rasel</t>
+          <t>Nazmin Akter</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>school corrected to Uttar Kattali Alhaz Mostofa Hakim High School (by user)</t>
+          <t>school corrected to Railway public High School (by user)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>3446</v>
+        <v>3507</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>মোহাম্মদ নুরুল ইসলাম</t>
+          <t>Mohiuddin Rasel</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>written in Bangla (kept as entered)</t>
+          <t>school corrected to Uttar Kattali Alhaz Mostofa Hakim High School (by user)</t>
         </is>
       </c>
     </row>
@@ -17520,12 +17520,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>ডাঃ খাস্তগীর সরকারি বালিকা উচ্চ বিদ্যালয়</t>
+          <t>মোহাম্মদ নুরুল ইসলাম</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -17536,7 +17536,7 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>3509</v>
+        <v>3446</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -17545,7 +17545,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>ফুলকি সহজপাঠ বিদ্যালয়</t>
+          <t>ডাঃ খাস্তগীর সরকারি বালিকা উচ্চ বিদ্যালয়</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -17556,16 +17556,16 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>3604</v>
+        <v>3509</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>মোঃ আনোয়ার হোসেন</t>
+          <t>ফুলকি সহজপাঠ বিদ্যালয়</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -17580,12 +17580,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>হালিশহর ক্যান্টনম্যান্ট পাবলিক স্কুল এন্ড কলেজ</t>
+          <t>মোঃ আনোয়ার হোসেন</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -17596,16 +17596,16 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>3639</v>
+        <v>3604</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>মোঃ আবু সায়েম</t>
+          <t>হালিশহর ক্যান্টনম্যান্ট পাবলিক স্কুল এন্ড কলেজ</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -17620,12 +17620,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>বিএএফ শাহীন কলেজ</t>
+          <t>মোঃ আবু সায়েম</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -17636,16 +17636,16 @@
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>3642</v>
+        <v>3639</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>মনির হোসেন</t>
+          <t>বিএএফ শাহীন কলেজ</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -17660,12 +17660,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>বিএএফ শাহীন কলেজ</t>
+          <t>মনির হোসেন</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -17676,16 +17676,16 @@
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>3643</v>
+        <v>3642</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>মো: রেজাউল করিম</t>
+          <t>বিএএফ শাহীন কলেজ</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -17700,12 +17700,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>বিএএফ শাহীন কলেজ</t>
+          <t>মো: রেজাউল করিম</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -17716,16 +17716,16 @@
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>3649</v>
+        <v>3643</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>মোঃ নিজাম উদ্দিন</t>
+          <t>বিএএফ শাহীন কলেজ</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -17740,12 +17740,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>বাংলাদেশ নৌবাহিনী স্কুল এন্ড কলেজ, চট্টগ্রাম</t>
+          <t>মোঃ নিজাম উদ্দিন</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -17756,16 +17756,16 @@
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>3670</v>
+        <v>3649</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>জুলফিকার আলী মিঠু</t>
+          <t>বাংলাদেশ নৌবাহিনী স্কুল এন্ড কলেজ, চট্টগ্রাম</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -17780,12 +17780,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>বিএএফ শাহীন কলেজ</t>
+          <t>জুলফিকার আলী মিঠু</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -17796,7 +17796,7 @@
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>3680</v>
+        <v>3670</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -17805,7 +17805,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>বলুয়ারদীঘি সিটি কর্পোরেশন বালিকা উচ্চ বিদ্যালয়</t>
+          <t>বিএএফ শাহীন কলেজ</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -17816,16 +17816,16 @@
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>3697</v>
+        <v>3680</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>কাকন চক্রবর্তী</t>
+          <t>বলুয়ারদীঘি সিটি কর্পোরেশন বালিকা উচ্চ বিদ্যালয়</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -17840,12 +17840,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>মুসলিম এডুকেশন সোসাইটি উচ্চ বিদ্যালয়</t>
+          <t>কাকন চক্রবর্তী</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -17856,16 +17856,16 @@
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>3718</v>
+        <v>3697</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>মনির আহমদ</t>
+          <t>মুসলিম এডুকেশন সোসাইটি উচ্চ বিদ্যালয়</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -17880,12 +17880,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>হাটহাজারী আনোয়ারুল উলুম নোমানীয়া ফাজিল মাদ্রাসা</t>
+          <t>মনির আহমদ</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -17896,16 +17896,16 @@
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>3724</v>
+        <v>3718</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>মনিরুল হক</t>
+          <t>হাটহাজারী আনোয়ারুল উলুম নোমানীয়া ফাজিল মাদ্রাসা</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -17920,12 +17920,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>বাহমনিখীল সরকারি প্রাথমিক বিদ্যালয়</t>
+          <t>মনিরুল হক</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -17936,16 +17936,16 @@
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>3748</v>
+        <v>3724</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>আবু বক্কর সিদ্দিক</t>
+          <t>বাহমনিখীল সরকারি প্রাথমিক বিদ্যালয়</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -17960,12 +17960,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>হালিশহর ক্যান্টনমেন্ট পাবলিক স্কুল এন্ড কলেজ</t>
+          <t>আবু বক্কর সিদ্দিক</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -17976,16 +17976,16 @@
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>3770</v>
+        <v>3748</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>মোহাম্মদ রেজাউল করিম</t>
+          <t>হালিশহর ক্যান্টনমেন্ট পাবলিক স্কুল এন্ড কলেজ</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -18000,12 +18000,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>রেলওয়ে পাবলিক স্কুল এন্ড কলেজ</t>
+          <t>মোহাম্মদ রেজাউল করিম</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -18016,16 +18016,16 @@
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>3773</v>
+        <v>3770</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>মোহাম্মদ রেজাউল করিম</t>
+          <t>রেলওয়ে পাবলিক স্কুল এন্ড কলেজ</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -18040,12 +18040,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>সেন্ট্রাল পাবলিক স্কুল এন্ড কলেজ</t>
+          <t>মোহাম্মদ রেজাউল করিম</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -18056,16 +18056,16 @@
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>3796</v>
+        <v>3773</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>মোহাম্মদ নওশাদ ইকবাল</t>
+          <t>সেন্ট্রাল পাবলিক স্কুল এন্ড কলেজ</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -18080,12 +18080,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>ইস্পাহানি পাবলিক স্কুল এন্ড কলেজ, চট্টগ্রাম।</t>
+          <t>মোহাম্মদ নওশাদ ইকবাল</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -18096,16 +18096,16 @@
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>3797</v>
+        <v>3796</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>মোহাম্মদ নওশাদ ইকবাল</t>
+          <t>ইস্পাহানি পাবলিক স্কুল এন্ড কলেজ, চট্টগ্রাম।</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -18120,12 +18120,12 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>ইস্পাহানি পাবলিক স্কুল এন্ড কলেজ, চট্টগ্রাম।</t>
+          <t>মোহাম্মদ নওশাদ ইকবাল</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -18136,16 +18136,16 @@
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>3835</v>
+        <v>3797</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>মো ইউসুফ</t>
+          <t>ইস্পাহানি পাবলিক স্কুল এন্ড কলেজ, চট্টগ্রাম।</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -18160,12 +18160,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>সি এম পি স্কুল এন্ড কলেজ</t>
+          <t>মো ইউসুফ</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -18176,16 +18176,16 @@
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>3840</v>
+        <v>3835</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>শাহা জাহান</t>
+          <t>সি এম পি স্কুল এন্ড কলেজ</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -18200,12 +18200,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>বাকলিয়া আদর্শ বালিকা উচ্চ বিদ্যালয়</t>
+          <t>শাহা জাহান</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -18216,26 +18216,46 @@
     </row>
     <row r="51">
       <c r="A51" t="n">
+        <v>3840</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Name of School</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>বাকলিয়া আদর্শ বালিকা উচ্চ বিদ্যালয়</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>written in Bangla (kept as entered)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
         <v>3846</v>
       </c>
-      <c r="B51" t="inlineStr">
+      <c r="B52" t="inlineStr">
         <is>
           <t>Name of School</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr">
+      <c r="C52" t="inlineStr">
         <is>
           <t>মোঃ আরিফুল ইসলাম</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr">
+      <c r="D52" t="inlineStr">
         <is>
           <t>written in Bangla (kept as entered)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D51"/>
+  <autoFilter ref="A1:D52"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Correct student, father and school for roll 11126020 (order 3667)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Admit_Card_Data_2026.xlsx
+++ b/Admit_Card_Data_2026.xlsx
@@ -16,7 +16,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Admit_Data'!$A$1:$M$285</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Separate'!$A$1:$N$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Review'!$A$1:$D$52</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Review'!$A$1:$D$54</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Centre_Map'!$A$1:$C$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Raw_Data'!$A$1:$S$286</definedName>
   </definedNames>
@@ -8977,17 +8977,17 @@
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>Nazmin Akter</t>
+          <t>Md.Naquibuddin</t>
         </is>
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>Nazmin Akter</t>
+          <t>Md.Jashim Uddin</t>
         </is>
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>Railway public High School</t>
+          <t>Railway Public High School</t>
         </is>
       </c>
       <c r="H147" t="n">
@@ -17203,7 +17203,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D52"/>
+  <dimension ref="A1:D54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -17296,27 +17296,27 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>3600</v>
+        <v>3667</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Mobile (Online)</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>0183519086</t>
+          <t>Nazmin Akter</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>invalid mobile (10 digits); replaced with Bkash number +8801835190860</t>
+          <t>father's name corrected to Md.Jashim Uddin (by user)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>3534</v>
+        <v>3600</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -17325,18 +17325,18 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>101812378354</t>
+          <t>0183519086</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>invalid mobile (12 digits); replaced with Bkash number +8801812378354</t>
+          <t>invalid mobile (10 digits); replaced with Bkash number +8801835190860</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>3648</v>
+        <v>3534</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -17345,58 +17345,58 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>017418691933</t>
+          <t>101812378354</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>invalid mobile (12 digits); replaced with Nagad Number +8801819315767 - different number, please confirm</t>
+          <t>invalid mobile (12 digits); replaced with Bkash number +8801812378354</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>3843</v>
+        <v>3648</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Student</t>
+          <t>Mobile (Online)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Safwan Zaman Ahnaf</t>
+          <t>017418691933</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>likely same student as order 3561 - kept, marked in file name</t>
+          <t>invalid mobile (12 digits); replaced with Nagad Number +8801819315767 - different number, please confirm</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>3795</v>
+        <v>3843</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Name (English)</t>
+          <t>Student</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>M. Jahirul Islam</t>
+          <t>Safwan Zaman Ahnaf</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>name corrected to Miskatul Jannat Labiba (by user)</t>
+          <t>likely same student as order 3561 - kept, marked in file name</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>3578</v>
+        <v>3667</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -17405,98 +17405,98 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Hossain Mohiuddin</t>
+          <t>Nazmin Akter</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>name corrected to Sarah Nur Shawli (by user)</t>
+          <t>name corrected to Md.Naquibuddin (by user)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>3750</v>
+        <v>3795</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Student</t>
+          <t>Name (English)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>MOHAMMED MUHTASIM ISLAM</t>
+          <t>M. Jahirul Islam</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>same student as order 3506 - kept both, marked in file name</t>
+          <t>name corrected to Miskatul Jannat Labiba (by user)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>3506</v>
+        <v>3578</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Student</t>
+          <t>Name (English)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>MOHAMMED MUHTASIM ISLAM</t>
+          <t>Hossain Mohiuddin</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>same student as order 3750 - kept both, marked in file name</t>
+          <t>name corrected to Sarah Nur Shawli (by user)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>3846</v>
+        <v>3750</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Student</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>মোঃ আরিফুল ইসলাম</t>
+          <t>MOHAMMED MUHTASIM ISLAM</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>school corrected to Chattogram Collegiate School (by user)</t>
+          <t>same student as order 3506 - kept both, marked in file name</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>3667</v>
+        <v>3506</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Student</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Nazmin Akter</t>
+          <t>MOHAMMED MUHTASIM ISLAM</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>school corrected to Railway public High School (by user)</t>
+          <t>same student as order 3750 - kept both, marked in file name</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>3507</v>
+        <v>3846</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -17505,38 +17505,38 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Mohiuddin Rasel</t>
+          <t>মোঃ আরিফুল ইসলাম</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>school corrected to Uttar Kattali Alhaz Mostofa Hakim High School (by user)</t>
+          <t>school corrected to Chattogram Collegiate School (by user)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>3446</v>
+        <v>3667</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>মোহাম্মদ নুরুল ইসলাম</t>
+          <t>Nazmin Akter</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>written in Bangla (kept as entered)</t>
+          <t>school corrected to Railway Public High School (by user)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>3446</v>
+        <v>3507</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -17545,27 +17545,27 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>ডাঃ খাস্তগীর সরকারি বালিকা উচ্চ বিদ্যালয়</t>
+          <t>Mohiuddin Rasel</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>written in Bangla (kept as entered)</t>
+          <t>school corrected to Uttar Kattali Alhaz Mostofa Hakim High School (by user)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>3509</v>
+        <v>3446</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>ফুলকি সহজপাঠ বিদ্যালয়</t>
+          <t>মোহাম্মদ নুরুল ইসলাম</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -17576,16 +17576,16 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>3604</v>
+        <v>3446</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>মোঃ আনোয়ার হোসেন</t>
+          <t>ডাঃ খাস্তগীর সরকারি বালিকা উচ্চ বিদ্যালয়</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -17596,7 +17596,7 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>3604</v>
+        <v>3509</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -17605,7 +17605,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>হালিশহর ক্যান্টনম্যান্ট পাবলিক স্কুল এন্ড কলেজ</t>
+          <t>ফুলকি সহজপাঠ বিদ্যালয়</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -17616,7 +17616,7 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>3639</v>
+        <v>3604</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -17625,7 +17625,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>মোঃ আবু সায়েম</t>
+          <t>মোঃ আনোয়ার হোসেন</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -17636,7 +17636,7 @@
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>3639</v>
+        <v>3604</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -17645,7 +17645,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>বিএএফ শাহীন কলেজ</t>
+          <t>হালিশহর ক্যান্টনম্যান্ট পাবলিক স্কুল এন্ড কলেজ</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -17656,7 +17656,7 @@
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>3642</v>
+        <v>3639</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -17665,7 +17665,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>মনির হোসেন</t>
+          <t>মোঃ আবু সায়েম</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -17676,7 +17676,7 @@
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>3642</v>
+        <v>3639</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -17696,7 +17696,7 @@
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>3643</v>
+        <v>3642</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -17705,7 +17705,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>মো: রেজাউল করিম</t>
+          <t>মনির হোসেন</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -17716,7 +17716,7 @@
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>3643</v>
+        <v>3642</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -17736,7 +17736,7 @@
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>3649</v>
+        <v>3643</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -17745,7 +17745,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>মোঃ নিজাম উদ্দিন</t>
+          <t>মো: রেজাউল করিম</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -17756,7 +17756,7 @@
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>3649</v>
+        <v>3643</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -17765,7 +17765,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>বাংলাদেশ নৌবাহিনী স্কুল এন্ড কলেজ, চট্টগ্রাম</t>
+          <t>বিএএফ শাহীন কলেজ</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -17776,7 +17776,7 @@
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>3670</v>
+        <v>3649</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -17785,7 +17785,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>জুলফিকার আলী মিঠু</t>
+          <t>মোঃ নিজাম উদ্দিন</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -17796,7 +17796,7 @@
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>3670</v>
+        <v>3649</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -17805,7 +17805,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>বিএএফ শাহীন কলেজ</t>
+          <t>বাংলাদেশ নৌবাহিনী স্কুল এন্ড কলেজ, চট্টগ্রাম</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -17816,16 +17816,16 @@
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>3680</v>
+        <v>3670</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Name of School</t>
+          <t>Fathers Name</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>বলুয়ারদীঘি সিটি কর্পোরেশন বালিকা উচ্চ বিদ্যালয়</t>
+          <t>জুলফিকার আলী মিঠু</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -17836,16 +17836,16 @@
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>3697</v>
+        <v>3670</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Fathers Name</t>
+          <t>Name of School</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>কাকন চক্রবর্তী</t>
+          <t>বিএএফ শাহীন কলেজ</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -17856,7 +17856,7 @@
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>3697</v>
+        <v>3680</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -17865,7 +17865,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>মুসলিম এডুকেশন সোসাইটি উচ্চ বিদ্যালয়</t>
+          <t>বলুয়ারদীঘি সিটি কর্পোরেশন বালিকা উচ্চ বিদ্যালয়</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -17876,7 +17876,7 @@
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>3718</v>
+        <v>3697</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -17885,7 +17885,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>মনির আহমদ</t>
+          <t>কাকন চক্রবর্তী</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -17896,7 +17896,7 @@
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>3718</v>
+        <v>3697</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -17905,7 +17905,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>হাটহাজারী আনোয়ারুল উলুম নোমানীয়া ফাজিল মাদ্রাসা</t>
+          <t>মুসলিম এডুকেশন সোসাইটি উচ্চ বিদ্যালয়</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -17916,7 +17916,7 @@
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>3724</v>
+        <v>3718</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -17925,7 +17925,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>মনিরুল হক</t>
+          <t>মনির আহমদ</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -17936,7 +17936,7 @@
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>3724</v>
+        <v>3718</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -17945,7 +17945,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>বাহমনিখীল সরকারি প্রাথমিক বিদ্যালয়</t>
+          <t>হাটহাজারী আনোয়ারুল উলুম নোমানীয়া ফাজিল মাদ্রাসা</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -17956,7 +17956,7 @@
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>3748</v>
+        <v>3724</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -17965,7 +17965,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>আবু বক্কর সিদ্দিক</t>
+          <t>মনিরুল হক</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -17976,7 +17976,7 @@
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>3748</v>
+        <v>3724</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -17985,7 +17985,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>হালিশহর ক্যান্টনমেন্ট পাবলিক স্কুল এন্ড কলেজ</t>
+          <t>বাহমনিখীল সরকারি প্রাথমিক বিদ্যালয়</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -17996,7 +17996,7 @@
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>3770</v>
+        <v>3748</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -18005,7 +18005,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>মোহাম্মদ রেজাউল করিম</t>
+          <t>আবু বক্কর সিদ্দিক</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -18016,7 +18016,7 @@
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>3770</v>
+        <v>3748</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -18025,7 +18025,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>রেলওয়ে পাবলিক স্কুল এন্ড কলেজ</t>
+          <t>হালিশহর ক্যান্টনমেন্ট পাবলিক স্কুল এন্ড কলেজ</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -18036,7 +18036,7 @@
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>3773</v>
+        <v>3770</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -18056,7 +18056,7 @@
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>3773</v>
+        <v>3770</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -18065,7 +18065,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>সেন্ট্রাল পাবলিক স্কুল এন্ড কলেজ</t>
+          <t>রেলওয়ে পাবলিক স্কুল এন্ড কলেজ</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -18076,7 +18076,7 @@
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>3796</v>
+        <v>3773</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -18085,7 +18085,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>মোহাম্মদ নওশাদ ইকবাল</t>
+          <t>মোহাম্মদ রেজাউল করিম</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -18096,7 +18096,7 @@
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>3796</v>
+        <v>3773</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
@@ -18105,7 +18105,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>ইস্পাহানি পাবলিক স্কুল এন্ড কলেজ, চট্টগ্রাম।</t>
+          <t>সেন্ট্রাল পাবলিক স্কুল এন্ড কলেজ</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -18116,7 +18116,7 @@
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>3797</v>
+        <v>3796</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
@@ -18136,7 +18136,7 @@
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>3797</v>
+        <v>3796</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
@@ -18156,7 +18156,7 @@
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>3835</v>
+        <v>3797</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
@@ -18165,7 +18165,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>মো ইউসুফ</t>
+          <t>মোহাম্মদ নওশাদ ইকবাল</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -18176,7 +18176,7 @@
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>3835</v>
+        <v>3797</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
@@ -18185,7 +18185,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>সি এম পি স্কুল এন্ড কলেজ</t>
+          <t>ইস্পাহানি পাবলিক স্কুল এন্ড কলেজ, চট্টগ্রাম।</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -18196,7 +18196,7 @@
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>3840</v>
+        <v>3835</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
@@ -18205,7 +18205,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>শাহা জাহান</t>
+          <t>মো ইউসুফ</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -18216,7 +18216,7 @@
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>3840</v>
+        <v>3835</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
@@ -18225,7 +18225,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>বাকলিয়া আদর্শ বালিকা উচ্চ বিদ্যালয়</t>
+          <t>সি এম পি স্কুল এন্ড কলেজ</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -18236,26 +18236,66 @@
     </row>
     <row r="52">
       <c r="A52" t="n">
+        <v>3840</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Fathers Name</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>শাহা জাহান</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>written in Bangla (kept as entered)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>3840</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Name of School</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>বাকলিয়া আদর্শ বালিকা উচ্চ বিদ্যালয়</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>written in Bangla (kept as entered)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
         <v>3846</v>
       </c>
-      <c r="B52" t="inlineStr">
+      <c r="B54" t="inlineStr">
         <is>
           <t>Name of School</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr">
+      <c r="C54" t="inlineStr">
         <is>
           <t>মোঃ আরিফুল ইসলাম</t>
         </is>
       </c>
-      <c r="D52" t="inlineStr">
+      <c r="D54" t="inlineStr">
         <is>
           <t>written in Bangla (kept as entered)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D52"/>
+  <autoFilter ref="A1:D54"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Order 3873: roll 64226024 (Class 6, centre 4); regenerate card
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Admit_Card_Data_2026.xlsx
+++ b/Admit_Card_Data_2026.xlsx
@@ -17788,12 +17788,12 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>54226024</t>
+          <t>64226024</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>Admit_54226024</t>
+          <t>Admit_64226024</t>
         </is>
       </c>
       <c r="D299" t="inlineStr">

</xml_diff>